<commit_message>
Complete rubric-compliant Colab experiments and submission
</commit_message>
<xml_diff>
--- a/submission_2A202602521/experiments.xlsx
+++ b/submission_2A202602521/experiments.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="1" r:id="R6c33b144d1314f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="2" r:id="R8fde531b8b934974"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seeds" sheetId="3" r:id="Rceb185df0c354aa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R60f5e3a4e9254fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="1" r:id="Rb0a4cc1ff3fc486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="2" r:id="Re715375283c4488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seeds" sheetId="3" r:id="Rb377b05a0f004fa7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rded9f8aa92604075"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,9 +18,9 @@
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="2">
     <x:numFmt numFmtId="164" formatCode="0.0000"/>
-    <x:numFmt numFmtId="200" formatCode="0.00"/>
+    <x:numFmt numFmtId="200" formatCode="0.000000"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -63,8 +63,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -84,6 +89,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F3864"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -114,7 +124,7 @@
     <x:xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <x:xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
@@ -233,14 +243,38 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="6">
@@ -1350,7 +1384,7 @@
   <x:cols>
     <x:col min="1" max="1" width="16" style="19" customWidth="1"/>
     <x:col min="2" max="2" width="11" style="19" customWidth="1"/>
-    <x:col min="3" max="3" width="34" style="19" customWidth="1"/>
+    <x:col min="3" max="3" width="55" style="19" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8" style="19" customWidth="1"/>
     <x:col min="5" max="5" width="15" style="19" customWidth="1"/>
     <x:col min="6" max="7" width="9" style="19" customWidth="1"/>
@@ -1368,7 +1402,7 @@
     <x:col min="23" max="23" width="10" style="19" customWidth="1"/>
     <x:col min="24" max="27" width="9" style="19" customWidth="1"/>
     <x:col min="28" max="28" width="22" style="19" customWidth="1"/>
-    <x:col min="29" max="29" width="36" style="19" customWidth="1"/>
+    <x:col min="29" max="29" width="72" style="19" hidden="0" customWidth="1"/>
     <x:col min="30" max="32" width="10" style="19" customWidth="1"/>
     <x:col min="33" max="33" width="9" style="19" customWidth="1"/>
   </x:cols>
@@ -1540,20 +1574,20 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="2" s="20" customFormat="1" ht="60" hidden="0" customHeight="1">
+    <x:row r="2" s="20" customFormat="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A2" s="32" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">base-s1</x:t>
+          <x:t xml:space="preserve">adam-lr0.0003</x:t>
         </x:is>
       </x:c>
       <x:c r="B2" s="32" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">baseline</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">M-base, AdamW lr=1e-3, He</x:t>
+          <x:t xml:space="preserve">optimizer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="48" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Adam/AdamW có thể hội tụ nhanh hơn SGD; thử cùng lưới lr cho từng optimizer và so lr tốt nhất.</x:t>
         </x:is>
       </x:c>
       <x:c r="D2" s="32" t="inlineStr">
@@ -1563,17 +1597,17 @@
       </x:c>
       <x:c r="E2" s="32" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adamw</x:t>
+          <x:t xml:space="preserve">adam</x:t>
         </x:is>
       </x:c>
       <x:c r="F2" s="33" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.0003</x:v>
       </x:c>
       <x:c r="G2" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H2" s="32" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I2" s="32" t="n">
         <x:v>20</x:v>
@@ -1608,45 +1642,41 @@
         <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q2" s="34" t="n">
-        <x:v>0.287590792568889</x:v>
+        <x:v>0.313508086585026</x:v>
       </x:c>
       <x:c r="R2" s="33" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="S2" s="34" t="n">
-        <x:v>0.2739207979441141</x:v>
+        <x:v>0.3012505951800551</x:v>
       </x:c>
       <x:c r="T2" s="34" t="n">
-        <x:v>0.287590792568889</x:v>
+        <x:v>0.313508086585026</x:v>
       </x:c>
       <x:c r="U2" s="34" t="n">
-        <x:v>0.8839310686086788</x:v>
+        <x:v>0.8726576450592716</x:v>
       </x:c>
       <x:c r="V2" s="34" t="n">
-        <x:v>0.8105385838093785</x:v>
-      </x:c>
-      <x:c r="W2" s="40" t="n">
-        <x:v>0.42669612695002</x:v>
-      </x:c>
-      <x:c r="X2" s="41" t="n">
-        <x:v>289.482421875</x:v>
+        <x:v>0.7877390598660482</x:v>
+      </x:c>
+      <x:c r="W2" s="49" t="n">
+        <x:v>1.498726749450003</x:v>
+      </x:c>
+      <x:c r="X2" s="49" t="n">
+        <x:v>160.77685546875</x:v>
       </x:c>
       <x:c r="Y2" s="33" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Z2" s="34" t="n">
-        <x:v>0.8835572231353752</x:v>
-      </x:c>
-      <x:c r="AA2" s="34" t="n">
-        <x:v>0.8118771210239729</x:v>
-      </x:c>
+      <x:c r="Z2" s="34" t="n"/>
+      <x:c r="AA2" s="34" t="n"/>
       <x:c r="AB2" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/base-s1.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC2" s="42" t="str">
-        <x:v>Rerun same seed for eval. Health: parameters=47879, logits=(20,7), gradients=True, overfit20_loss=0.00000439. Peak memory includes retained data from the first pass; not comparable across runs.</x:v>
+          <x:t xml:space="preserve">figures/adam-lr0.0003.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC2" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/adam-lr0.0003.json. Independent GPU process. grad_p90=1.108847; mean clip fraction=0.000000. Optimizer/lr tuned jointly; betas=.9/.999, eps=1e-8, wd=0; momentum=.9.</x:v>
       </x:c>
       <x:c r="AD2" s="35" t="n">
         <x:f>IF(P2="","",P2-LN(7))</x:f>
@@ -1654,31 +1684,31 @@
       </x:c>
       <x:c r="AE2" s="35" t="n">
         <x:f>IF(OR(T2="",S2=""),"",T2-S2)</x:f>
-        <x:v>0.013669994624774862</x:v>
+        <x:v>0.0122574914049709</x:v>
       </x:c>
       <x:c r="AF2" s="35" t="n">
         <x:f>IF(OR(V2="",Seeds!$C$8=""),"",V2-Seeds!$C$8)</x:f>
-        <x:v>-0.0000351346524984919</x:v>
+        <x:v>-0.06577127986220033</x:v>
       </x:c>
       <x:c r="AG2" s="35" t="str">
         <x:f>IF(OR(AF2="",Seeds!$C$10=""),"",IF(ABS(AF2)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Không</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+        <x:v>Có</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" s="20" customFormat="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A3" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">base-s2</x:t>
+          <x:t xml:space="preserve">adam-lr0.001</x:t>
         </x:is>
       </x:c>
       <x:c r="B3" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">baseline</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Baseline repeat, seed 2</x:t>
+          <x:t xml:space="preserve">optimizer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Adam/AdamW có thể hội tụ nhanh hơn SGD; thử cùng lưới lr cho từng optimizer và so lr tốt nhất.</x:t>
         </x:is>
       </x:c>
       <x:c r="D3" s="33" t="inlineStr">
@@ -1688,7 +1718,7 @@
       </x:c>
       <x:c r="E3" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adamw</x:t>
+          <x:t xml:space="preserve">adam</x:t>
         </x:is>
       </x:c>
       <x:c r="F3" s="33" t="n">
@@ -1698,7 +1728,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H3" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I3" s="33" t="n">
         <x:v>20</x:v>
@@ -1723,34 +1753,34 @@
         </x:is>
       </x:c>
       <x:c r="O3" s="33" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P3" s="34" t="n">
-        <x:v>1.978156701881548</x:v>
+        <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q3" s="34" t="n">
-        <x:v>0.2875723438817323</x:v>
+        <x:v>0.2494106242251538</x:v>
       </x:c>
       <x:c r="R3" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="S3" s="34" t="n">
-        <x:v>0.2738224057208951</x:v>
+        <x:v>0.2329071531352277</x:v>
       </x:c>
       <x:c r="T3" s="34" t="n">
-        <x:v>0.2875723438817323</x:v>
+        <x:v>0.2528524937388311</x:v>
       </x:c>
       <x:c r="U3" s="34" t="n">
-        <x:v>0.884587250704589</x:v>
+        <x:v>0.8993352122372582</x:v>
       </x:c>
       <x:c r="V3" s="34" t="n">
-        <x:v>0.8128493532287756</x:v>
-      </x:c>
-      <x:c r="W3" s="40" t="n">
-        <x:v>0.4248054920500181</x:v>
-      </x:c>
-      <x:c r="X3" s="41" t="n">
-        <x:v>161.318359375</x:v>
+        <x:v>0.845555844686964</x:v>
+      </x:c>
+      <x:c r="W3" s="49" t="n">
+        <x:v>1.468359294449993</x:v>
+      </x:c>
+      <x:c r="X3" s="49" t="n">
+        <x:v>160.77685546875</x:v>
       </x:c>
       <x:c r="Y3" s="33" t="b">
         <x:v>0</x:v>
@@ -1759,45 +1789,43 @@
       <x:c r="AA3" s="34" t="n"/>
       <x:c r="AB3" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/base-s2.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC3" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/adam-lr0.001.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC3" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/adam-lr0.001.json. Independent GPU process. grad_p90=1.250242; mean clip fraction=0.000000. Optimizer/lr tuned jointly; betas=.9/.999, eps=1e-8, wd=0; momentum=.9.</x:v>
       </x:c>
       <x:c r="AD3" s="35" t="n">
         <x:f>IF(P3="","",P3-LN(7))</x:f>
-        <x:v>0.03224655282623479</x:v>
+        <x:v>0.32315163933839863</x:v>
       </x:c>
       <x:c r="AE3" s="35" t="n">
         <x:f>IF(OR(T3="",S3=""),"",T3-S3)</x:f>
-        <x:v>0.013749938160837194</x:v>
+        <x:v>0.019945340603603423</x:v>
       </x:c>
       <x:c r="AF3" s="35" t="n">
         <x:f>IF(OR(V3="",Seeds!$C$8=""),"",V3-Seeds!$C$8)</x:f>
-        <x:v>0.0022756347668986265</x:v>
+        <x:v>-0.007954495041284537</x:v>
       </x:c>
       <x:c r="AG3" s="35" t="str">
         <x:f>IF(OR(AF3="",Seeds!$C$10=""),"",IF(ABS(AF3)&gt;Seeds!$C$10,"Có","Không"))</x:f>
         <x:v>Không</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+    <x:row r="4" s="20" customFormat="1" ht="48" hidden="0" customHeight="1">
       <x:c r="A4" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">base-s3</x:t>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
         </x:is>
       </x:c>
       <x:c r="B4" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">baseline</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Baseline repeat, seed 3</x:t>
+          <x:t xml:space="preserve">optimizer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Adam/AdamW có thể hội tụ nhanh hơn SGD; thử cùng lưới lr cho từng optimizer và so lr tốt nhất.</x:t>
         </x:is>
       </x:c>
       <x:c r="D4" s="33" t="inlineStr">
@@ -1807,17 +1835,17 @@
       </x:c>
       <x:c r="E4" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adamw</x:t>
+          <x:t xml:space="preserve">adam</x:t>
         </x:is>
       </x:c>
       <x:c r="F4" s="33" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.003</x:v>
       </x:c>
       <x:c r="G4" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H4" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I4" s="33" t="n">
         <x:v>20</x:v>
@@ -1842,81 +1870,83 @@
         </x:is>
       </x:c>
       <x:c r="O4" s="33" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P4" s="34" t="n">
-        <x:v>1.900539953068861</x:v>
+        <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q4" s="34" t="n">
-        <x:v>0.2934093584084592</x:v>
+        <x:v>0.2144964847657847</x:v>
       </x:c>
       <x:c r="R4" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="S4" s="34" t="n">
-        <x:v>0.2791241085778391</x:v>
+        <x:v>0.1869444217974311</x:v>
       </x:c>
       <x:c r="T4" s="34" t="n">
-        <x:v>0.2934093584084592</x:v>
+        <x:v>0.2159531313607559</x:v>
       </x:c>
       <x:c r="U4" s="34" t="n">
-        <x:v>0.8803489597900217</x:v>
+        <x:v>0.9152879671263527</x:v>
       </x:c>
       <x:c r="V4" s="34" t="n">
-        <x:v>0.8083332183474771</x:v>
-      </x:c>
-      <x:c r="W4" s="40" t="n">
-        <x:v>0.3979958650000128</x:v>
-      </x:c>
-      <x:c r="X4" s="41" t="n">
-        <x:v>161.50146484375</x:v>
+        <x:v>0.8677466182111557</x:v>
+      </x:c>
+      <x:c r="W4" s="49" t="n">
+        <x:v>1.466127746050006</x:v>
+      </x:c>
+      <x:c r="X4" s="49" t="n">
+        <x:v>160.77685546875</x:v>
       </x:c>
       <x:c r="Y4" s="33" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Z4" s="34" t="n"/>
-      <x:c r="AA4" s="34" t="n"/>
+      <x:c r="Z4" s="34" t="n">
+        <x:v>0.9140297582678588</x:v>
+      </x:c>
+      <x:c r="AA4" s="34" t="n">
+        <x:v>0.8699991815477335</x:v>
+      </x:c>
       <x:c r="AB4" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/base-s3.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC4" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/adam-lr0.003.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC4" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/adam-lr0.003.json. Independent GPU process. grad_p90=0.919864; mean clip fraction=0.000000. Optimizer/lr tuned jointly; betas=.9/.999, eps=1e-8, wd=0; momentum=.9. Selected by validation before scoring; per-class eval: Summary, eval_result.json.</x:v>
       </x:c>
       <x:c r="AD4" s="35" t="n">
         <x:f>IF(P4="","",P4-LN(7))</x:f>
-        <x:v>-0.04537019598645231</x:v>
+        <x:v>0.32315163933839863</x:v>
       </x:c>
       <x:c r="AE4" s="35" t="n">
         <x:f>IF(OR(T4="",S4=""),"",T4-S4)</x:f>
-        <x:v>0.014285249830620128</x:v>
+        <x:v>0.029008709563324797</x:v>
       </x:c>
       <x:c r="AF4" s="35" t="n">
         <x:f>IF(OR(V4="",Seeds!$C$8=""),"",V4-Seeds!$C$8)</x:f>
-        <x:v>-0.0022405001143999126</x:v>
+        <x:v>0.014236278482907205</x:v>
       </x:c>
       <x:c r="AG4" s="35" t="str">
         <x:f>IF(OR(AF4="",Seeds!$C$10=""),"",IF(ABS(AF4)&gt;Seeds!$C$10,"Có","Không"))</x:f>
         <x:v>Không</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+    <x:row r="5" s="20" customFormat="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A5" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">clip-highlr-1</x:t>
+          <x:t xml:space="preserve">adamw-lr0.0003</x:t>
         </x:is>
       </x:c>
       <x:c r="B5" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">clipping</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AdamW lr=0.01, clip norm 1</x:t>
+          <x:t xml:space="preserve">optimizer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Adam/AdamW có thể hội tụ nhanh hơn SGD; thử cùng lưới lr cho từng optimizer và so lr tốt nhất.</x:t>
         </x:is>
       </x:c>
       <x:c r="D5" s="33" t="inlineStr">
@@ -1930,13 +1960,13 @@
         </x:is>
       </x:c>
       <x:c r="F5" s="33" t="n">
-        <x:v>0.01</x:v>
+        <x:v>0.0003</x:v>
       </x:c>
       <x:c r="G5" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I5" s="33" t="n">
         <x:v>20</x:v>
@@ -1949,9 +1979,7 @@
       <x:c r="K5" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L5" s="33" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="L5" s="33" t="n"/>
       <x:c r="M5" s="33" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">fp32</x:t>
@@ -1969,28 +1997,28 @@
         <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q5" s="34" t="n">
-        <x:v>0.2229622221888631</x:v>
+        <x:v>0.313508086585026</x:v>
       </x:c>
       <x:c r="R5" s="33" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="S5" s="34" t="n">
-        <x:v>0.2022958104004091</x:v>
+        <x:v>0.3012505951800551</x:v>
       </x:c>
       <x:c r="T5" s="34" t="n">
-        <x:v>0.2257890115929425</x:v>
+        <x:v>0.313508086585026</x:v>
       </x:c>
       <x:c r="U5" s="34" t="n">
-        <x:v>0.9107592349562187</x:v>
+        <x:v>0.8726576450592716</x:v>
       </x:c>
       <x:c r="V5" s="34" t="n">
-        <x:v>0.8671875241333343</x:v>
-      </x:c>
-      <x:c r="W5" s="40" t="n">
-        <x:v>0.438121021850003</x:v>
-      </x:c>
-      <x:c r="X5" s="41" t="n">
-        <x:v>163.1494140625</x:v>
+        <x:v>0.7877390598660482</x:v>
+      </x:c>
+      <x:c r="W5" s="49" t="n">
+        <x:v>1.507558503849964</x:v>
+      </x:c>
+      <x:c r="X5" s="49" t="n">
+        <x:v>160.77685546875</x:v>
       </x:c>
       <x:c r="Y5" s="33" t="b">
         <x:v>0</x:v>
@@ -1999,13 +2027,11 @@
       <x:c r="AA5" s="34" t="n"/>
       <x:c r="AB5" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/clip-highlr-1.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC5" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/adamw-lr0.0003.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC5" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/adamw-lr0.0003.json. Independent GPU process. grad_p90=1.108847; mean clip fraction=0.000000. Optimizer/lr tuned jointly; betas=.9/.999, eps=1e-8, wd=0; momentum=.9.</x:v>
       </x:c>
       <x:c r="AD5" s="35" t="n">
         <x:f>IF(P5="","",P5-LN(7))</x:f>
@@ -2013,11 +2039,11 @@
       </x:c>
       <x:c r="AE5" s="35" t="n">
         <x:f>IF(OR(T5="",S5=""),"",T5-S5)</x:f>
-        <x:v>0.023493201192533425</x:v>
+        <x:v>0.0122574914049709</x:v>
       </x:c>
       <x:c r="AF5" s="35" t="n">
         <x:f>IF(OR(V5="",Seeds!$C$8=""),"",V5-Seeds!$C$8)</x:f>
-        <x:v>0.05661380567145735</x:v>
+        <x:v>-0.06577127986220033</x:v>
       </x:c>
       <x:c r="AG5" s="35" t="str">
         <x:f>IF(OR(AF5="",Seeds!$C$10=""),"",IF(ABS(AF5)&gt;Seeds!$C$10,"Có","Không"))</x:f>
@@ -2027,17 +2053,17 @@
     <x:row r="6" s="20" customFormat="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A6" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">clip-highlr-none</x:t>
+          <x:t xml:space="preserve">adamw-lr0.001</x:t>
         </x:is>
       </x:c>
       <x:c r="B6" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">clipping</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AdamW lr=0.01, no clipping</x:t>
+          <x:t xml:space="preserve">optimizer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Adam/AdamW có thể hội tụ nhanh hơn SGD; thử cùng lưới lr cho từng optimizer và so lr tốt nhất.</x:t>
         </x:is>
       </x:c>
       <x:c r="D6" s="33" t="inlineStr">
@@ -2051,13 +2077,13 @@
         </x:is>
       </x:c>
       <x:c r="F6" s="33" t="n">
-        <x:v>0.01</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="G6" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I6" s="33" t="n">
         <x:v>20</x:v>
@@ -2088,45 +2114,41 @@
         <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q6" s="34" t="n">
-        <x:v>0.2297001319570597</x:v>
+        <x:v>0.2494106242251538</x:v>
       </x:c>
       <x:c r="R6" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="S6" s="34" t="n">
-        <x:v>0.205611940140619</x:v>
+        <x:v>0.2329071531352277</x:v>
       </x:c>
       <x:c r="T6" s="34" t="n">
-        <x:v>0.2297001319570597</x:v>
+        <x:v>0.2528524937388311</x:v>
       </x:c>
       <x:c r="U6" s="34" t="n">
-        <x:v>0.9073922678083518</x:v>
+        <x:v>0.8993352122372582</x:v>
       </x:c>
       <x:c r="V6" s="34" t="n">
-        <x:v>0.8676104419728523</x:v>
-      </x:c>
-      <x:c r="W6" s="40" t="n">
-        <x:v>0.4219738436500052</x:v>
-      </x:c>
-      <x:c r="X6" s="41" t="n">
-        <x:v>289.66552734375</x:v>
+        <x:v>0.845555844686964</x:v>
+      </x:c>
+      <x:c r="W6" s="49" t="n">
+        <x:v>1.459386985249955</x:v>
+      </x:c>
+      <x:c r="X6" s="49" t="n">
+        <x:v>160.77685546875</x:v>
       </x:c>
       <x:c r="Y6" s="33" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Z6" s="34" t="n">
-        <x:v>0.9067666067141124</x:v>
-      </x:c>
-      <x:c r="AA6" s="34" t="n">
-        <x:v>0.8695424856379919</x:v>
-      </x:c>
+      <x:c r="Z6" s="34" t="n"/>
+      <x:c r="AA6" s="34" t="n"/>
       <x:c r="AB6" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/clip-highlr-none.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC6" s="42" t="str">
-        <x:v>Rerun same seed to recover weights for eval. Peak memory includes retained data from the first pass; not comparable across runs.</x:v>
+          <x:t xml:space="preserve">figures/adamw-lr0.001.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC6" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/adamw-lr0.001.json. Independent GPU process. grad_p90=1.250242; mean clip fraction=0.000000. Optimizer/lr tuned jointly; betas=.9/.999, eps=1e-8, wd=0; momentum=.9.</x:v>
       </x:c>
       <x:c r="AD6" s="35" t="n">
         <x:f>IF(P6="","",P6-LN(7))</x:f>
@@ -2134,31 +2156,31 @@
       </x:c>
       <x:c r="AE6" s="35" t="n">
         <x:f>IF(OR(T6="",S6=""),"",T6-S6)</x:f>
-        <x:v>0.0240881918164407</x:v>
+        <x:v>0.019945340603603423</x:v>
       </x:c>
       <x:c r="AF6" s="35" t="n">
         <x:f>IF(OR(V6="",Seeds!$C$8=""),"",V6-Seeds!$C$8)</x:f>
-        <x:v>0.05703672351097533</x:v>
+        <x:v>-0.007954495041284537</x:v>
       </x:c>
       <x:c r="AG6" s="35" t="str">
         <x:f>IF(OR(AF6="",Seeds!$C$10=""),"",IF(ABS(AF6)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Có</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" s="20" customFormat="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A7" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">dropout-p03</x:t>
+          <x:t xml:space="preserve">adamw-lr0.003</x:t>
         </x:is>
       </x:c>
       <x:c r="B7" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">dropout</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Dropout p=0.3</x:t>
+          <x:t xml:space="preserve">optimizer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Adam/AdamW có thể hội tụ nhanh hơn SGD; thử cùng lưới lr cho từng optimizer và so lr tốt nhất.</x:t>
         </x:is>
       </x:c>
       <x:c r="D7" s="33" t="inlineStr">
@@ -2172,13 +2194,13 @@
         </x:is>
       </x:c>
       <x:c r="F7" s="33" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.003</x:v>
       </x:c>
       <x:c r="G7" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I7" s="33" t="n">
         <x:v>20</x:v>
@@ -2189,7 +2211,7 @@
         </x:is>
       </x:c>
       <x:c r="K7" s="33" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L7" s="33" t="n"/>
       <x:c r="M7" s="33" t="inlineStr">
@@ -2209,28 +2231,28 @@
         <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q7" s="34" t="n">
-        <x:v>0.3649630790420414</x:v>
+        <x:v>0.2144964847657847</x:v>
       </x:c>
       <x:c r="R7" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="S7" s="34" t="n">
-        <x:v>0.3601284161028007</x:v>
+        <x:v>0.1869444217974311</x:v>
       </x:c>
       <x:c r="T7" s="34" t="n">
-        <x:v>0.3649630790420414</x:v>
+        <x:v>0.2159531313607559</x:v>
       </x:c>
       <x:c r="U7" s="34" t="n">
-        <x:v>0.8495944579505604</x:v>
+        <x:v>0.9152879671263527</x:v>
       </x:c>
       <x:c r="V7" s="34" t="n">
-        <x:v>0.7495524199248325</x:v>
-      </x:c>
-      <x:c r="W7" s="40" t="n">
-        <x:v>0.4236440889999983</x:v>
-      </x:c>
-      <x:c r="X7" s="41" t="n">
-        <x:v>162.783203125</x:v>
+        <x:v>0.8677466182111557</x:v>
+      </x:c>
+      <x:c r="W7" s="49" t="n">
+        <x:v>1.476678678500036</x:v>
+      </x:c>
+      <x:c r="X7" s="49" t="n">
+        <x:v>160.77685546875</x:v>
       </x:c>
       <x:c r="Y7" s="33" t="b">
         <x:v>0</x:v>
@@ -2239,13 +2261,11 @@
       <x:c r="AA7" s="34" t="n"/>
       <x:c r="AB7" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/dropout-p03.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC7" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/adamw-lr0.003.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC7" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/adamw-lr0.003.json. Independent GPU process. grad_p90=0.919864; mean clip fraction=0.000000. Optimizer/lr tuned jointly; betas=.9/.999, eps=1e-8, wd=0; momentum=.9.</x:v>
       </x:c>
       <x:c r="AD7" s="35" t="n">
         <x:f>IF(P7="","",P7-LN(7))</x:f>
@@ -2253,31 +2273,31 @@
       </x:c>
       <x:c r="AE7" s="35" t="n">
         <x:f>IF(OR(T7="",S7=""),"",T7-S7)</x:f>
-        <x:v>0.004834662939240675</x:v>
+        <x:v>0.029008709563324797</x:v>
       </x:c>
       <x:c r="AF7" s="35" t="n">
         <x:f>IF(OR(V7="",Seeds!$C$8=""),"",V7-Seeds!$C$8)</x:f>
-        <x:v>-0.06102129853704452</x:v>
+        <x:v>0.014236278482907205</x:v>
       </x:c>
       <x:c r="AG7" s="35" t="str">
         <x:f>IF(OR(AF7="",Seeds!$C$10=""),"",IF(ABS(AF7)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Có</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" s="20" customFormat="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A8" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">init-normal</x:t>
+          <x:t xml:space="preserve">base-s1</x:t>
         </x:is>
       </x:c>
       <x:c r="B8" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">initialization</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Normal N(0, 0.01) initialization</x:t>
+          <x:t xml:space="preserve">baseline</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SGD momentum: lr thấp học chậm, lr cao có thể dao động; chọn lr bằng F1 val tại epoch min val loss.</x:t>
         </x:is>
       </x:c>
       <x:c r="D8" s="33" t="inlineStr">
@@ -2287,17 +2307,17 @@
       </x:c>
       <x:c r="E8" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adamw</x:t>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
         </x:is>
       </x:c>
       <x:c r="F8" s="33" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="G8" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I8" s="33" t="n">
         <x:v>20</x:v>
@@ -2318,85 +2338,87 @@
       </x:c>
       <x:c r="N8" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">normal</x:t>
+          <x:t xml:space="preserve">he</x:t>
         </x:is>
       </x:c>
       <x:c r="O8" s="33" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="P8" s="34" t="n">
-        <x:v>1.945995658844474</x:v>
+        <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q8" s="34" t="n">
-        <x:v>0.3738819723969875</x:v>
+        <x:v>0.2379235743460702</x:v>
       </x:c>
       <x:c r="R8" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="S8" s="34" t="n">
-        <x:v>0.3662302778480211</x:v>
+        <x:v>0.2208534015460324</x:v>
       </x:c>
       <x:c r="T8" s="34" t="n">
-        <x:v>0.3738819723969875</x:v>
+        <x:v>0.2425536006353739</x:v>
       </x:c>
       <x:c r="U8" s="34" t="n">
-        <x:v>0.8457003937092575</x:v>
+        <x:v>0.9053806931864633</x:v>
       </x:c>
       <x:c r="V8" s="34" t="n">
-        <x:v>0.7561769579452472</x:v>
-      </x:c>
-      <x:c r="W8" s="40" t="n">
-        <x:v>0.4280980429500119</x:v>
-      </x:c>
-      <x:c r="X8" s="41" t="n">
-        <x:v>163.8818359375</x:v>
+        <x:v>0.8390357563558714</x:v>
+      </x:c>
+      <x:c r="W8" s="49" t="n">
+        <x:v>1.308921133550001</x:v>
+      </x:c>
+      <x:c r="X8" s="49" t="n">
+        <x:v>160.59375</x:v>
       </x:c>
       <x:c r="Y8" s="33" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Z8" s="34" t="n"/>
-      <x:c r="AA8" s="34" t="n"/>
+      <x:c r="Z8" s="34" t="n">
+        <x:v>0.9033415660525116</x:v>
+      </x:c>
+      <x:c r="AA8" s="34" t="n">
+        <x:v>0.8409922038067058</x:v>
+      </x:c>
       <x:c r="AB8" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/init-normal.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC8" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/base-s1.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC8" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/base-s1.json. Independent GPU process. grad_p90=0.696241; mean clip fraction=0.000000. Health and eval per-class values: Summary A20:F51, health_checks.json/eval_baseline.json.</x:v>
       </x:c>
       <x:c r="AD8" s="35" t="n">
         <x:f>IF(P8="","",P8-LN(7))</x:f>
-        <x:v>0.0000855097891607759</x:v>
+        <x:v>0.32315163933839863</x:v>
       </x:c>
       <x:c r="AE8" s="35" t="n">
         <x:f>IF(OR(T8="",S8=""),"",T8-S8)</x:f>
-        <x:v>0.0076516945489664145</x:v>
+        <x:v>0.02170019908934151</x:v>
       </x:c>
       <x:c r="AF8" s="35" t="n">
         <x:f>IF(OR(V8="",Seeds!$C$8=""),"",V8-Seeds!$C$8)</x:f>
-        <x:v>-0.05439676051662978</x:v>
+        <x:v>-0.01447458337237717</x:v>
       </x:c>
       <x:c r="AG8" s="35" t="str">
         <x:f>IF(OR(AF8="",Seeds!$C$10=""),"",IF(ABS(AF8)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Có</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A9" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">init-xavier</x:t>
+          <x:t xml:space="preserve">base-s2</x:t>
         </x:is>
       </x:c>
       <x:c r="B9" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">initialization</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Xavier normal initialization</x:t>
+          <x:t xml:space="preserve">baseline</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SGD momentum: lr thấp học chậm, lr cao có thể dao động; chọn lr bằng F1 val tại epoch min val loss.</x:t>
         </x:is>
       </x:c>
       <x:c r="D9" s="33" t="inlineStr">
@@ -2406,17 +2428,17 @@
       </x:c>
       <x:c r="E9" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adamw</x:t>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
         </x:is>
       </x:c>
       <x:c r="F9" s="33" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="G9" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I9" s="33" t="n">
         <x:v>20</x:v>
@@ -2437,38 +2459,38 @@
       </x:c>
       <x:c r="N9" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">xavier</x:t>
+          <x:t xml:space="preserve">he</x:t>
         </x:is>
       </x:c>
       <x:c r="O9" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="P9" s="34" t="n">
-        <x:v>2.022176189935135</x:v>
+        <x:v>1.978156701881548</x:v>
       </x:c>
       <x:c r="Q9" s="34" t="n">
-        <x:v>0.3003156890183035</x:v>
+        <x:v>0.2278535272960154</x:v>
       </x:c>
       <x:c r="R9" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="S9" s="34" t="n">
-        <x:v>0.2885334570805709</x:v>
+        <x:v>0.2075339349080401</x:v>
       </x:c>
       <x:c r="T9" s="34" t="n">
-        <x:v>0.3003156890183035</x:v>
+        <x:v>0.2325465058975711</x:v>
       </x:c>
       <x:c r="U9" s="34" t="n">
-        <x:v>0.8782835997504357</x:v>
+        <x:v>0.9099847249413739</x:v>
       </x:c>
       <x:c r="V9" s="34" t="n">
-        <x:v>0.8038252517683885</x:v>
-      </x:c>
-      <x:c r="W9" s="40" t="n">
-        <x:v>0.411226255899993</x:v>
-      </x:c>
-      <x:c r="X9" s="41" t="n">
-        <x:v>163.69873046875</x:v>
+        <x:v>0.860050003346835</x:v>
+      </x:c>
+      <x:c r="W9" s="49" t="n">
+        <x:v>1.37662679904999</x:v>
+      </x:c>
+      <x:c r="X9" s="49" t="n">
+        <x:v>160.59375</x:v>
       </x:c>
       <x:c r="Y9" s="33" t="b">
         <x:v>0</x:v>
@@ -2477,65 +2499,63 @@
       <x:c r="AA9" s="34" t="n"/>
       <x:c r="AB9" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/init-xavier.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC9" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/base-s2.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC9" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/base-s2.json. Independent GPU process. grad_p90=0.666963; mean clip fraction=0.000000.</x:v>
       </x:c>
       <x:c r="AD9" s="35" t="n">
         <x:f>IF(P9="","",P9-LN(7))</x:f>
-        <x:v>0.07626604087982192</x:v>
+        <x:v>0.03224655282623479</x:v>
       </x:c>
       <x:c r="AE9" s="35" t="n">
         <x:f>IF(OR(T9="",S9=""),"",T9-S9)</x:f>
-        <x:v>0.011782231937732646</x:v>
+        <x:v>0.025012570989530997</x:v>
       </x:c>
       <x:c r="AF9" s="35" t="n">
         <x:f>IF(OR(V9="",Seeds!$C$8=""),"",V9-Seeds!$C$8)</x:f>
-        <x:v>-0.006748466693488497</x:v>
+        <x:v>0.006539663618586489</x:v>
       </x:c>
       <x:c r="AG9" s="35" t="str">
         <x:f>IF(OR(AF9="",Seeds!$C$10=""),"",IF(ABS(AF9)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Có</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A10" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">loss-mse</x:t>
+          <x:t xml:space="preserve">base-s3</x:t>
         </x:is>
       </x:c>
       <x:c r="B10" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">loss</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MSE on one-hot labels</x:t>
+          <x:t xml:space="preserve">baseline</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SGD momentum: lr thấp học chậm, lr cao có thể dao động; chọn lr bằng F1 val tại epoch min val loss.</x:t>
         </x:is>
       </x:c>
       <x:c r="D10" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">mse</x:t>
+          <x:t xml:space="preserve">ce</x:t>
         </x:is>
       </x:c>
       <x:c r="E10" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adamw</x:t>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
         </x:is>
       </x:c>
       <x:c r="F10" s="33" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="G10" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H10" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I10" s="33" t="n">
         <x:v>20</x:v>
@@ -2560,34 +2580,34 @@
         </x:is>
       </x:c>
       <x:c r="O10" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="P10" s="34" t="n">
-        <x:v>0.6358503211013448</x:v>
+        <x:v>1.900539953068861</x:v>
       </x:c>
       <x:c r="Q10" s="34" t="n">
-        <x:v>0.02882067333352126</x:v>
+        <x:v>0.2276589681332745</x:v>
       </x:c>
       <x:c r="R10" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="S10" s="34" t="n">
-        <x:v>0.02787003503057877</x:v>
+        <x:v>0.2158851095926004</x:v>
       </x:c>
       <x:c r="T10" s="34" t="n">
-        <x:v>0.02882067333352126</x:v>
+        <x:v>0.2375198889177752</x:v>
       </x:c>
       <x:c r="U10" s="34" t="n">
-        <x:v>0.8743465071749748</x:v>
+        <x:v>0.9091026440911341</x:v>
       </x:c>
       <x:c r="V10" s="34" t="n">
-        <x:v>0.7590204129234761</x:v>
-      </x:c>
-      <x:c r="W10" s="40" t="n">
-        <x:v>0.4261545501999933</x:v>
-      </x:c>
-      <x:c r="X10" s="41" t="n">
-        <x:v>161.71533203125</x:v>
+        <x:v>0.861445259482039</x:v>
+      </x:c>
+      <x:c r="W10" s="49" t="n">
+        <x:v>1.359536895699989</x:v>
+      </x:c>
+      <x:c r="X10" s="49" t="n">
+        <x:v>160.59375</x:v>
       </x:c>
       <x:c r="Y10" s="33" t="b">
         <x:v>0</x:v>
@@ -2596,35 +2616,33 @@
       <x:c r="AA10" s="34" t="n"/>
       <x:c r="AB10" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/loss-mse.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC10" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/base-s3.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC10" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/base-s3.json. Independent GPU process. grad_p90=0.709586; mean clip fraction=0.000000.</x:v>
       </x:c>
       <x:c r="AD10" s="35" t="n">
         <x:f>IF(P10="","",P10-LN(7))</x:f>
-        <x:v>-1.3100598279539684</x:v>
+        <x:v>-0.04537019598645231</x:v>
       </x:c>
       <x:c r="AE10" s="35" t="n">
         <x:f>IF(OR(T10="",S10=""),"",T10-S10)</x:f>
-        <x:v>0.0009506383029424907</x:v>
+        <x:v>0.021634779325174797</x:v>
       </x:c>
       <x:c r="AF10" s="35" t="n">
         <x:f>IF(OR(V10="",Seeds!$C$8=""),"",V10-Seeds!$C$8)</x:f>
-        <x:v>-0.05155330553840087</x:v>
+        <x:v>0.00793491975379046</x:v>
       </x:c>
       <x:c r="AG10" s="35" t="str">
         <x:f>IF(OR(AF10="",Seeds!$C$10=""),"",IF(ABS(AF10)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Có</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A11" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">lr-adamw-3e4</x:t>
+          <x:t xml:space="preserve">batch2048</x:t>
         </x:is>
       </x:c>
       <x:c r="B11" s="33" t="inlineStr">
@@ -2632,9 +2650,9 @@
           <x:t xml:space="preserve">hyperparameter</x:t>
         </x:is>
       </x:c>
-      <x:c r="C11" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AdamW, lower learning rate</x:t>
+      <x:c r="C11" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Batch 2048 giảm số bước/epoch bốn lần so batch 512, có thể làm học chậm với lr giữ nguyên.</x:t>
         </x:is>
       </x:c>
       <x:c r="D11" s="33" t="inlineStr">
@@ -2644,11 +2662,11 @@
       </x:c>
       <x:c r="E11" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adamw</x:t>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
         </x:is>
       </x:c>
       <x:c r="F11" s="33" t="n">
-        <x:v>0.0003</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="G11" s="33" t="n">
         <x:v>0</x:v>
@@ -2685,28 +2703,28 @@
         <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q11" s="34" t="n">
-        <x:v>0.3774216148970816</x:v>
+        <x:v>0.2810376736596674</x:v>
       </x:c>
       <x:c r="R11" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="S11" s="34" t="n">
-        <x:v>0.3687890330728893</x:v>
+        <x:v>0.2753028769605783</x:v>
       </x:c>
       <x:c r="T11" s="34" t="n">
-        <x:v>0.3774216148970816</x:v>
+        <x:v>0.291032188046048</x:v>
       </x:c>
       <x:c r="U11" s="34" t="n">
-        <x:v>0.8458402357952712</x:v>
+        <x:v>0.8851788902992621</x:v>
       </x:c>
       <x:c r="V11" s="34" t="n">
-        <x:v>0.7347919884872669</x:v>
-      </x:c>
-      <x:c r="W11" s="40" t="n">
-        <x:v>0.4170817043499938</x:v>
-      </x:c>
-      <x:c r="X11" s="41" t="n">
-        <x:v>162.60009765625</x:v>
+        <x:v>0.7969625312167096</x:v>
+      </x:c>
+      <x:c r="W11" s="49" t="n">
+        <x:v>0.3896035869499769</x:v>
+      </x:c>
+      <x:c r="X11" s="49" t="n">
+        <x:v>160.8125</x:v>
       </x:c>
       <x:c r="Y11" s="33" t="b">
         <x:v>0</x:v>
@@ -2715,13 +2733,11 @@
       <x:c r="AA11" s="34" t="n"/>
       <x:c r="AB11" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/lr-adamw-3e4.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC11" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/batch2048.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC11" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/batch2048.json. Independent GPU process. grad_p90=1.114660; mean clip fraction=0.000000.</x:v>
       </x:c>
       <x:c r="AD11" s="35" t="n">
         <x:f>IF(P11="","",P11-LN(7))</x:f>
@@ -2729,31 +2745,31 @@
       </x:c>
       <x:c r="AE11" s="35" t="n">
         <x:f>IF(OR(T11="",S11=""),"",T11-S11)</x:f>
-        <x:v>0.008632581824192298</x:v>
+        <x:v>0.01572931108546971</x:v>
       </x:c>
       <x:c r="AF11" s="35" t="n">
         <x:f>IF(OR(V11="",Seeds!$C$8=""),"",V11-Seeds!$C$8)</x:f>
-        <x:v>-0.07578172997461008</x:v>
+        <x:v>-0.056547808511538955</x:v>
       </x:c>
       <x:c r="AG11" s="35" t="str">
         <x:f>IF(OR(AF11="",Seeds!$C$10=""),"",IF(ABS(AF11)&gt;Seeds!$C$10,"Có","Không"))</x:f>
         <x:v>Có</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+    <x:row r="12" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">opt-adam-lr1e3</x:t>
+          <x:t xml:space="preserve">clip-normal</x:t>
         </x:is>
       </x:c>
       <x:c r="B12" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">optimizer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Adam, lr=1e-3</x:t>
+          <x:t xml:space="preserve">clipping</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">lr gấp 10 có thể gây dao động; clip ở phân vị 90 gradient baseline có thể giảm bước cực lớn, không chắc cứu được phân kỳ.</x:t>
         </x:is>
       </x:c>
       <x:c r="D12" s="33" t="inlineStr">
@@ -2763,17 +2779,17 @@
       </x:c>
       <x:c r="E12" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adam</x:t>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
         </x:is>
       </x:c>
       <x:c r="F12" s="33" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="G12" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H12" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I12" s="33" t="n">
         <x:v>20</x:v>
@@ -2786,7 +2802,9 @@
       <x:c r="K12" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L12" s="33" t="n"/>
+      <x:c r="L12" s="33" t="n">
+        <x:v>0.6962409436702729</x:v>
+      </x:c>
       <x:c r="M12" s="33" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">fp32</x:t>
@@ -2804,28 +2822,28 @@
         <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q12" s="34" t="n">
-        <x:v>0.287590792568889</x:v>
+        <x:v>0.2426736448028664</x:v>
       </x:c>
       <x:c r="R12" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="S12" s="34" t="n">
-        <x:v>0.2739207979441141</x:v>
+        <x:v>0.2228872693967651</x:v>
       </x:c>
       <x:c r="T12" s="34" t="n">
-        <x:v>0.287590792568889</x:v>
+        <x:v>0.2460131979330264</x:v>
       </x:c>
       <x:c r="U12" s="34" t="n">
-        <x:v>0.8839310686086788</x:v>
+        <x:v>0.9026914223015856</x:v>
       </x:c>
       <x:c r="V12" s="34" t="n">
-        <x:v>0.8105385838093785</x:v>
-      </x:c>
-      <x:c r="W12" s="40" t="n">
-        <x:v>0.4230451794000146</x:v>
-      </x:c>
-      <x:c r="X12" s="41" t="n">
-        <x:v>162.4169921875</x:v>
+        <x:v>0.8441129852605526</x:v>
+      </x:c>
+      <x:c r="W12" s="49" t="n">
+        <x:v>1.324455269500038</x:v>
+      </x:c>
+      <x:c r="X12" s="49" t="n">
+        <x:v>160.59375</x:v>
       </x:c>
       <x:c r="Y12" s="33" t="b">
         <x:v>0</x:v>
@@ -2834,13 +2852,11 @@
       <x:c r="AA12" s="34" t="n"/>
       <x:c r="AB12" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/opt-adam-lr1e3.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC12" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/clip-normal.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC12" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/clip-normal.json. Independent GPU process. grad_p90=0.722627; mean clip fraction=0.133356.</x:v>
       </x:c>
       <x:c r="AD12" s="35" t="n">
         <x:f>IF(P12="","",P12-LN(7))</x:f>
@@ -2848,31 +2864,31 @@
       </x:c>
       <x:c r="AE12" s="35" t="n">
         <x:f>IF(OR(T12="",S12=""),"",T12-S12)</x:f>
-        <x:v>0.013669994624774862</x:v>
+        <x:v>0.023125928536261303</x:v>
       </x:c>
       <x:c r="AF12" s="35" t="n">
         <x:f>IF(OR(V12="",Seeds!$C$8=""),"",V12-Seeds!$C$8)</x:f>
-        <x:v>-0.0000351346524984919</x:v>
+        <x:v>-0.009397354467695962</x:v>
       </x:c>
       <x:c r="AG12" s="35" t="str">
         <x:f>IF(OR(AF12="",Seeds!$C$10=""),"",IF(ABS(AF12)&gt;Seeds!$C$10,"Có","Không"))</x:f>
         <x:v>Không</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+    <x:row r="13" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A13" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">opt-adam-lr3e4</x:t>
+          <x:t xml:space="preserve">dropout-p03</x:t>
         </x:is>
       </x:c>
       <x:c r="B13" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">optimizer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C13" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Adam, lr=3e-4</x:t>
+          <x:t xml:space="preserve">dropout</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">p=0.3 có thể giảm train-val gap nhưng giảm F1 nếu mạng chưa overfit.</x:t>
         </x:is>
       </x:c>
       <x:c r="D13" s="33" t="inlineStr">
@@ -2882,17 +2898,17 @@
       </x:c>
       <x:c r="E13" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adam</x:t>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
         </x:is>
       </x:c>
       <x:c r="F13" s="33" t="n">
-        <x:v>0.0003</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="G13" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H13" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I13" s="33" t="n">
         <x:v>20</x:v>
@@ -2903,7 +2919,7 @@
         </x:is>
       </x:c>
       <x:c r="K13" s="33" t="n">
-        <x:v>0</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="L13" s="33" t="n"/>
       <x:c r="M13" s="33" t="inlineStr">
@@ -2923,28 +2939,28 @@
         <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q13" s="34" t="n">
-        <x:v>0.3774216148970816</x:v>
+        <x:v>0.3150786634582124</x:v>
       </x:c>
       <x:c r="R13" s="33" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="S13" s="34" t="n">
-        <x:v>0.3687890330728893</x:v>
+        <x:v>0.3085967255391667</x:v>
       </x:c>
       <x:c r="T13" s="34" t="n">
-        <x:v>0.3774216148970816</x:v>
+        <x:v>0.3150786634582124</x:v>
       </x:c>
       <x:c r="U13" s="34" t="n">
-        <x:v>0.8458402357952712</x:v>
+        <x:v>0.8727867300617457</x:v>
       </x:c>
       <x:c r="V13" s="34" t="n">
-        <x:v>0.7347919884872669</x:v>
-      </x:c>
-      <x:c r="W13" s="40" t="n">
-        <x:v>0.4099446818999979</x:v>
-      </x:c>
-      <x:c r="X13" s="41" t="n">
-        <x:v>162.23388671875</x:v>
+        <x:v>0.7874882114860531</x:v>
+      </x:c>
+      <x:c r="W13" s="49" t="n">
+        <x:v>1.442498998099984</x:v>
+      </x:c>
+      <x:c r="X13" s="49" t="n">
+        <x:v>160.59375</x:v>
       </x:c>
       <x:c r="Y13" s="33" t="b">
         <x:v>0</x:v>
@@ -2953,13 +2969,11 @@
       <x:c r="AA13" s="34" t="n"/>
       <x:c r="AB13" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/opt-adam-lr3e4.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC13" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/dropout-p03.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC13" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/dropout-p03.json. Independent GPU process. grad_p90=0.397102; mean clip fraction=0.000000.</x:v>
       </x:c>
       <x:c r="AD13" s="35" t="n">
         <x:f>IF(P13="","",P13-LN(7))</x:f>
@@ -2967,31 +2981,31 @@
       </x:c>
       <x:c r="AE13" s="35" t="n">
         <x:f>IF(OR(T13="",S13=""),"",T13-S13)</x:f>
-        <x:v>0.008632581824192298</x:v>
+        <x:v>0.006481937919045666</x:v>
       </x:c>
       <x:c r="AF13" s="35" t="n">
         <x:f>IF(OR(V13="",Seeds!$C$8=""),"",V13-Seeds!$C$8)</x:f>
-        <x:v>-0.07578172997461008</x:v>
+        <x:v>-0.06602212824219544</x:v>
       </x:c>
       <x:c r="AG13" s="35" t="str">
         <x:f>IF(OR(AF13="",Seeds!$C$10=""),"",IF(ABS(AF13)&gt;Seeds!$C$10,"Có","Không"))</x:f>
         <x:v>Có</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+    <x:row r="14" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">opt-sgdm-lr01</x:t>
+          <x:t xml:space="preserve">final-s2</x:t>
         </x:is>
       </x:c>
       <x:c r="B14" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">optimizer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C14" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SGD momentum, lr=0.01</x:t>
+          <x:t xml:space="preserve">other</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Fixed validation-selected config repeated for noise; no retuning.</x:t>
         </x:is>
       </x:c>
       <x:c r="D14" s="33" t="inlineStr">
@@ -3001,17 +3015,17 @@
       </x:c>
       <x:c r="E14" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">sgd_momentum</x:t>
+          <x:t xml:space="preserve">adam</x:t>
         </x:is>
       </x:c>
       <x:c r="F14" s="33" t="n">
-        <x:v>0.01</x:v>
+        <x:v>0.003</x:v>
       </x:c>
       <x:c r="G14" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H14" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I14" s="33" t="n">
         <x:v>20</x:v>
@@ -3036,34 +3050,34 @@
         </x:is>
       </x:c>
       <x:c r="O14" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="P14" s="34" t="n">
-        <x:v>2.269061788393712</x:v>
+        <x:v>1.978156701881548</x:v>
       </x:c>
       <x:c r="Q14" s="34" t="n">
-        <x:v>0.4384593225403088</x:v>
+        <x:v>0.2098134267899787</x:v>
       </x:c>
       <x:c r="R14" s="33" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="S14" s="34" t="n">
-        <x:v>0.4320220136821856</x:v>
+        <x:v>0.1819792724782051</x:v>
       </x:c>
       <x:c r="T14" s="34" t="n">
-        <x:v>0.4384593225403088</x:v>
+        <x:v>0.2098134267899787</x:v>
       </x:c>
       <x:c r="U14" s="34" t="n">
-        <x:v>0.8159463006389708</x:v>
+        <x:v>0.9172242421634647</x:v>
       </x:c>
       <x:c r="V14" s="34" t="n">
-        <x:v>0.6616020830040074</x:v>
-      </x:c>
-      <x:c r="W14" s="40" t="n">
-        <x:v>0.3874024855999892</x:v>
-      </x:c>
-      <x:c r="X14" s="41" t="n">
-        <x:v>161.6845703125</x:v>
+        <x:v>0.86256369796698</x:v>
+      </x:c>
+      <x:c r="W14" s="49" t="n">
+        <x:v>1.477861961750011</x:v>
+      </x:c>
+      <x:c r="X14" s="49" t="n">
+        <x:v>160.77685546875</x:v>
       </x:c>
       <x:c r="Y14" s="33" t="b">
         <x:v>0</x:v>
@@ -3072,45 +3086,43 @@
       <x:c r="AA14" s="34" t="n"/>
       <x:c r="AB14" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/opt-sgdm-lr01.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC14" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/final-s2.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC14" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/final-s2.json. Independent GPU process. grad_p90=0.857768; mean clip fraction=0.000000.</x:v>
       </x:c>
       <x:c r="AD14" s="35" t="n">
         <x:f>IF(P14="","",P14-LN(7))</x:f>
-        <x:v>0.32315163933839863</x:v>
+        <x:v>0.03224655282623479</x:v>
       </x:c>
       <x:c r="AE14" s="35" t="n">
         <x:f>IF(OR(T14="",S14=""),"",T14-S14)</x:f>
-        <x:v>0.0064373088581231586</x:v>
+        <x:v>0.02783415431177358</x:v>
       </x:c>
       <x:c r="AF14" s="35" t="n">
         <x:f>IF(OR(V14="",Seeds!$C$8=""),"",V14-Seeds!$C$8)</x:f>
-        <x:v>-0.14897163545786962</x:v>
+        <x:v>0.009053358238731435</x:v>
       </x:c>
       <x:c r="AG14" s="35" t="str">
         <x:f>IF(OR(AF14="",Seeds!$C$10=""),"",IF(ABS(AF14)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Có</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">opt-sgdm-lr05</x:t>
+          <x:t xml:space="preserve">final-s3</x:t>
         </x:is>
       </x:c>
       <x:c r="B15" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">optimizer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C15" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SGD momentum, lr=0.05</x:t>
+          <x:t xml:space="preserve">other</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Fixed validation-selected config repeated for noise; no retuning.</x:t>
         </x:is>
       </x:c>
       <x:c r="D15" s="33" t="inlineStr">
@@ -3120,17 +3132,17 @@
       </x:c>
       <x:c r="E15" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">sgd_momentum</x:t>
+          <x:t xml:space="preserve">adam</x:t>
         </x:is>
       </x:c>
       <x:c r="F15" s="33" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.003</x:v>
       </x:c>
       <x:c r="G15" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H15" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I15" s="33" t="n">
         <x:v>20</x:v>
@@ -3155,34 +3167,34 @@
         </x:is>
       </x:c>
       <x:c r="O15" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="P15" s="34" t="n">
-        <x:v>2.269061788393712</x:v>
+        <x:v>1.900539953068861</x:v>
       </x:c>
       <x:c r="Q15" s="34" t="n">
-        <x:v>0.3171317149623301</x:v>
+        <x:v>0.2152615206158666</x:v>
       </x:c>
       <x:c r="R15" s="33" t="n">
         <x:v>19</x:v>
       </x:c>
       <x:c r="S15" s="34" t="n">
-        <x:v>0.320164991355389</x:v>
+        <x:v>0.1920850317411504</x:v>
       </x:c>
       <x:c r="T15" s="34" t="n">
-        <x:v>0.3321563509947277</x:v>
+        <x:v>0.2195941316663664</x:v>
       </x:c>
       <x:c r="U15" s="34" t="n">
-        <x:v>0.8697424754200641</x:v>
+        <x:v>0.9158688496374863</x:v>
       </x:c>
       <x:c r="V15" s="34" t="n">
-        <x:v>0.766244743482292</x:v>
-      </x:c>
-      <x:c r="W15" s="40" t="n">
-        <x:v>0.3705713885000194</x:v>
-      </x:c>
-      <x:c r="X15" s="41" t="n">
-        <x:v>161.86767578125</x:v>
+        <x:v>0.8718252825287924</x:v>
+      </x:c>
+      <x:c r="W15" s="49" t="n">
+        <x:v>1.477130472949989</x:v>
+      </x:c>
+      <x:c r="X15" s="49" t="n">
+        <x:v>160.77685546875</x:v>
       </x:c>
       <x:c r="Y15" s="33" t="b">
         <x:v>0</x:v>
@@ -3191,45 +3203,43 @@
       <x:c r="AA15" s="34" t="n"/>
       <x:c r="AB15" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/opt-sgdm-lr05.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC15" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/final-s3.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC15" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/final-s3.json. Independent GPU process. grad_p90=0.885323; mean clip fraction=0.000000.</x:v>
       </x:c>
       <x:c r="AD15" s="35" t="n">
         <x:f>IF(P15="","",P15-LN(7))</x:f>
-        <x:v>0.32315163933839863</x:v>
+        <x:v>-0.04537019598645231</x:v>
       </x:c>
       <x:c r="AE15" s="35" t="n">
         <x:f>IF(OR(T15="",S15=""),"",T15-S15)</x:f>
-        <x:v>0.011991359639338672</x:v>
+        <x:v>0.027509099925215996</x:v>
       </x:c>
       <x:c r="AF15" s="35" t="n">
         <x:f>IF(OR(V15="",Seeds!$C$8=""),"",V15-Seeds!$C$8)</x:f>
-        <x:v>-0.04432897497958499</x:v>
+        <x:v>0.01831494280054391</x:v>
       </x:c>
       <x:c r="AG15" s="35" t="str">
         <x:f>IF(OR(AF15="",Seeds!$C$10=""),"",IF(ABS(AF15)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Có</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" s="20" customFormat="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A16" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">precision-bf16</x:t>
+          <x:t xml:space="preserve">highlr-clip</x:t>
         </x:is>
       </x:c>
       <x:c r="B16" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">mixed_precision</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BF16 requested; CPU falls back to FP32</x:t>
+          <x:t xml:space="preserve">clipping</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">lr gấp 10 có thể gây dao động; clip ở phân vị 90 gradient baseline có thể giảm bước cực lớn, không chắc cứu được phân kỳ.</x:t>
         </x:is>
       </x:c>
       <x:c r="D16" s="33" t="inlineStr">
@@ -3239,17 +3249,17 @@
       </x:c>
       <x:c r="E16" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adamw</x:t>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
         </x:is>
       </x:c>
       <x:c r="F16" s="33" t="n">
-        <x:v>0.001</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G16" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H16" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I16" s="33" t="n">
         <x:v>20</x:v>
@@ -3262,10 +3272,12 @@
       <x:c r="K16" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L16" s="33" t="n"/>
+      <x:c r="L16" s="33" t="n">
+        <x:v>0.6962409436702729</x:v>
+      </x:c>
       <x:c r="M16" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">bf16</x:t>
+          <x:t xml:space="preserve">fp32</x:t>
         </x:is>
       </x:c>
       <x:c r="N16" s="33" t="inlineStr">
@@ -3280,28 +3292,28 @@
         <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q16" s="34" t="n">
-        <x:v>0.2883216216286628</x:v>
+        <x:v>0.3084116313413428</x:v>
       </x:c>
       <x:c r="R16" s="33" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="S16" s="34" t="n">
-        <x:v>0.2759269311369999</x:v>
+        <x:v>0.2862392416991544</x:v>
       </x:c>
       <x:c r="T16" s="34" t="n">
-        <x:v>0.2883216216286628</x:v>
+        <x:v>0.3084116313413428</x:v>
       </x:c>
       <x:c r="U16" s="34" t="n">
-        <x:v>0.8846948215399841</x:v>
+        <x:v>0.8859426432305674</x:v>
       </x:c>
       <x:c r="V16" s="34" t="n">
-        <x:v>0.8121172525672452</x:v>
-      </x:c>
-      <x:c r="W16" s="40" t="n">
-        <x:v>0.4716468666999845</x:v>
-      </x:c>
-      <x:c r="X16" s="41" t="n">
-        <x:v>163.33251953125</x:v>
+        <x:v>0.802701640920526</x:v>
+      </x:c>
+      <x:c r="W16" s="49" t="n">
+        <x:v>1.310327988150004</x:v>
+      </x:c>
+      <x:c r="X16" s="49" t="n">
+        <x:v>160.59375</x:v>
       </x:c>
       <x:c r="Y16" s="33" t="b">
         <x:v>0</x:v>
@@ -3310,13 +3322,11 @@
       <x:c r="AA16" s="34" t="n"/>
       <x:c r="AB16" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/precision-bf16.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC16" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/highlr-clip.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC16" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/highlr-clip.json. Independent GPU process. grad_p90=0.293581; mean clip fraction=0.001032. Compare highlr-none at same lr; relative to baseline lr/clip both change.</x:v>
       </x:c>
       <x:c r="AD16" s="35" t="n">
         <x:f>IF(P16="","",P16-LN(7))</x:f>
@@ -3324,31 +3334,31 @@
       </x:c>
       <x:c r="AE16" s="35" t="n">
         <x:f>IF(OR(T16="",S16=""),"",T16-S16)</x:f>
-        <x:v>0.012394690491662919</x:v>
+        <x:v>0.022172389642188428</x:v>
       </x:c>
       <x:c r="AF16" s="35" t="n">
         <x:f>IF(OR(V16="",Seeds!$C$8=""),"",V16-Seeds!$C$8)</x:f>
-        <x:v>0.0015435341053682272</x:v>
+        <x:v>-0.05080869880772254</x:v>
       </x:c>
       <x:c r="AG16" s="35" t="str">
         <x:f>IF(OR(AF16="",Seeds!$C$10=""),"",IF(ABS(AF16)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Không</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
+        <x:v>Có</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A17" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">precision-fp16</x:t>
+          <x:t xml:space="preserve">highlr-none</x:t>
         </x:is>
       </x:c>
       <x:c r="B17" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">mixed_precision</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" s="33" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FP16 mixed precision on Tesla T4</x:t>
+          <x:t xml:space="preserve">clipping</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">lr gấp 10 có thể gây dao động; clip ở phân vị 90 gradient baseline có thể giảm bước cực lớn, không chắc cứu được phân kỳ.</x:t>
         </x:is>
       </x:c>
       <x:c r="D17" s="33" t="inlineStr">
@@ -3358,17 +3368,17 @@
       </x:c>
       <x:c r="E17" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">adamw</x:t>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
         </x:is>
       </x:c>
       <x:c r="F17" s="33" t="n">
-        <x:v>0.001</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G17" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H17" s="33" t="n">
-        <x:v>2048</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I17" s="33" t="n">
         <x:v>20</x:v>
@@ -3384,7 +3394,7 @@
       <x:c r="L17" s="33" t="n"/>
       <x:c r="M17" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">fp16</x:t>
+          <x:t xml:space="preserve">fp32</x:t>
         </x:is>
       </x:c>
       <x:c r="N17" s="33" t="inlineStr">
@@ -3399,28 +3409,28 @@
         <x:v>2.269061788393712</x:v>
       </x:c>
       <x:c r="Q17" s="34" t="n">
-        <x:v>0.2875404350523853</x:v>
+        <x:v>0.3334942100785721</x:v>
       </x:c>
       <x:c r="R17" s="33" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="S17" s="34" t="n">
-        <x:v>0.2740928982840851</x:v>
+        <x:v>0.3530189502608768</x:v>
       </x:c>
       <x:c r="T17" s="34" t="n">
-        <x:v>0.2875404350523853</x:v>
+        <x:v>0.3708138307793944</x:v>
       </x:c>
       <x:c r="U17" s="34" t="n">
-        <x:v>0.884544222370431</x:v>
+        <x:v>0.8662464232697231</x:v>
       </x:c>
       <x:c r="V17" s="34" t="n">
-        <x:v>0.8127790715003889</x:v>
-      </x:c>
-      <x:c r="W17" s="40" t="n">
-        <x:v>0.5496686643500027</x:v>
-      </x:c>
-      <x:c r="X17" s="41" t="n">
-        <x:v>163.5166015625</x:v>
+        <x:v>0.7731754847049565</x:v>
+      </x:c>
+      <x:c r="W17" s="49" t="n">
+        <x:v>1.312749423249966</x:v>
+      </x:c>
+      <x:c r="X17" s="49" t="n">
+        <x:v>160.59375</x:v>
       </x:c>
       <x:c r="Y17" s="33" t="b">
         <x:v>0</x:v>
@@ -3429,13 +3439,11 @@
       <x:c r="AA17" s="34" t="n"/>
       <x:c r="AB17" s="33" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">figures/precision-fp16.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="AC17" s="42" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+          <x:t xml:space="preserve">figures/highlr-none.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC17" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/highlr-none.json. Independent GPU process. grad_p90=0.303937; mean clip fraction=0.000000.</x:v>
       </x:c>
       <x:c r="AD17" s="35" t="n">
         <x:f>IF(P17="","",P17-LN(7))</x:f>
@@ -3443,402 +3451,1068 @@
       </x:c>
       <x:c r="AE17" s="35" t="n">
         <x:f>IF(OR(T17="",S17=""),"",T17-S17)</x:f>
-        <x:v>0.013447536768300183</x:v>
+        <x:v>0.017794880518517575</x:v>
       </x:c>
       <x:c r="AF17" s="35" t="n">
         <x:f>IF(OR(V17="",Seeds!$C$8=""),"",V17-Seeds!$C$8)</x:f>
-        <x:v>0.0022053530385118814</x:v>
+        <x:v>-0.08033485502329207</x:v>
       </x:c>
       <x:c r="AG17" s="35" t="str">
         <x:f>IF(OR(AF17="",Seeds!$C$10=""),"",IF(ABS(AF17)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-        <x:v>Không</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A18" s="33" t="n"/>
-      <x:c r="B18" s="33" t="n"/>
-      <x:c r="C18" s="33" t="n"/>
-      <x:c r="D18" s="33" t="n"/>
-      <x:c r="E18" s="33" t="n"/>
-      <x:c r="F18" s="33" t="n"/>
-      <x:c r="G18" s="33" t="n"/>
-      <x:c r="H18" s="33" t="n"/>
-      <x:c r="I18" s="33" t="n"/>
-      <x:c r="J18" s="33" t="n"/>
-      <x:c r="K18" s="33" t="n"/>
+        <x:v>Có</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A18" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">init-normal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">initialization</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">He giữ tín hiệu qua ReLU tốt hơn normal nhỏ; zeros không phá đối xứng và gradient hidden bằng 0.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E18" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F18" s="33" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G18" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="33" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I18" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J18" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">256-128</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K18" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L18" s="33" t="n"/>
-      <x:c r="M18" s="33" t="n"/>
-      <x:c r="N18" s="33" t="n"/>
-      <x:c r="O18" s="33" t="n"/>
-      <x:c r="P18" s="34" t="n"/>
-      <x:c r="Q18" s="34" t="n"/>
-      <x:c r="R18" s="33" t="n"/>
-      <x:c r="S18" s="34" t="n"/>
-      <x:c r="T18" s="34" t="n"/>
-      <x:c r="U18" s="34" t="n"/>
-      <x:c r="V18" s="34" t="n"/>
-      <x:c r="W18" s="33" t="n"/>
-      <x:c r="X18" s="33" t="n"/>
-      <x:c r="Y18" s="33" t="n"/>
+      <x:c r="M18" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">fp32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N18" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">normal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O18" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P18" s="34" t="n">
+        <x:v>1.945995658844474</x:v>
+      </x:c>
+      <x:c r="Q18" s="34" t="n">
+        <x:v>0.2339697460492089</x:v>
+      </x:c>
+      <x:c r="R18" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="S18" s="34" t="n">
+        <x:v>0.2125945053431124</x:v>
+      </x:c>
+      <x:c r="T18" s="34" t="n">
+        <x:v>0.2339697460492089</x:v>
+      </x:c>
+      <x:c r="U18" s="34" t="n">
+        <x:v>0.9046276973386975</x:v>
+      </x:c>
+      <x:c r="V18" s="34" t="n">
+        <x:v>0.8449007627822941</x:v>
+      </x:c>
+      <x:c r="W18" s="49" t="n">
+        <x:v>1.305649247450015</x:v>
+      </x:c>
+      <x:c r="X18" s="49" t="n">
+        <x:v>160.59375</x:v>
+      </x:c>
+      <x:c r="Y18" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z18" s="34" t="n"/>
       <x:c r="AA18" s="34" t="n"/>
-      <x:c r="AB18" s="33" t="n"/>
-      <x:c r="AC18" s="33" t="n"/>
-      <x:c r="AD18" s="35" t="str">
+      <x:c r="AB18" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">figures/init-normal.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC18" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/init-normal.json. Independent GPU process. grad_p90=0.748205; mean clip fraction=0.000000.</x:v>
+      </x:c>
+      <x:c r="AD18" s="35" t="n">
         <x:f>IF(P18="","",P18-LN(7))</x:f>
-      </x:c>
-      <x:c r="AE18" s="35" t="str">
+        <x:v>0.0000855097891607759</x:v>
+      </x:c>
+      <x:c r="AE18" s="35" t="n">
         <x:f>IF(OR(T18="",S18=""),"",T18-S18)</x:f>
-      </x:c>
-      <x:c r="AF18" s="35" t="str">
+        <x:v>0.021375240706096504</x:v>
+      </x:c>
+      <x:c r="AF18" s="35" t="n">
         <x:f>IF(OR(V18="",Seeds!$C$8=""),"",V18-Seeds!$C$8)</x:f>
+        <x:v>-0.008609576945954434</x:v>
       </x:c>
       <x:c r="AG18" s="35" t="str">
         <x:f>IF(OR(AF18="",Seeds!$C$10=""),"",IF(ABS(AF18)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="19" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A19" s="33" t="n"/>
-      <x:c r="B19" s="33" t="n"/>
-      <x:c r="C19" s="33" t="n"/>
-      <x:c r="D19" s="33" t="n"/>
-      <x:c r="E19" s="33" t="n"/>
-      <x:c r="F19" s="33" t="n"/>
-      <x:c r="G19" s="33" t="n"/>
-      <x:c r="H19" s="33" t="n"/>
-      <x:c r="I19" s="33" t="n"/>
-      <x:c r="J19" s="33" t="n"/>
-      <x:c r="K19" s="33" t="n"/>
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A19" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">init-xavier</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">initialization</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">He giữ tín hiệu qua ReLU tốt hơn normal nhỏ; zeros không phá đối xứng và gradient hidden bằng 0.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E19" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F19" s="33" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G19" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="33" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I19" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J19" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">256-128</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K19" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L19" s="33" t="n"/>
-      <x:c r="M19" s="33" t="n"/>
-      <x:c r="N19" s="33" t="n"/>
-      <x:c r="O19" s="33" t="n"/>
-      <x:c r="P19" s="34" t="n"/>
-      <x:c r="Q19" s="34" t="n"/>
-      <x:c r="R19" s="33" t="n"/>
-      <x:c r="S19" s="34" t="n"/>
-      <x:c r="T19" s="34" t="n"/>
-      <x:c r="U19" s="34" t="n"/>
-      <x:c r="V19" s="34" t="n"/>
-      <x:c r="W19" s="33" t="n"/>
-      <x:c r="X19" s="33" t="n"/>
-      <x:c r="Y19" s="33" t="n"/>
+      <x:c r="M19" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">fp32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N19" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">xavier</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O19" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P19" s="34" t="n">
+        <x:v>2.022176189935135</x:v>
+      </x:c>
+      <x:c r="Q19" s="34" t="n">
+        <x:v>0.2317417757264057</x:v>
+      </x:c>
+      <x:c r="R19" s="33" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="S19" s="34" t="n">
+        <x:v>0.215736884474663</x:v>
+      </x:c>
+      <x:c r="T19" s="34" t="n">
+        <x:v>0.2357558486809462</x:v>
+      </x:c>
+      <x:c r="U19" s="34" t="n">
+        <x:v>0.9072309115552591</x:v>
+      </x:c>
+      <x:c r="V19" s="34" t="n">
+        <x:v>0.8514344709948414</x:v>
+      </x:c>
+      <x:c r="W19" s="49" t="n">
+        <x:v>1.311863490699977</x:v>
+      </x:c>
+      <x:c r="X19" s="49" t="n">
+        <x:v>160.59375</x:v>
+      </x:c>
+      <x:c r="Y19" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z19" s="34" t="n"/>
       <x:c r="AA19" s="34" t="n"/>
-      <x:c r="AB19" s="33" t="n"/>
-      <x:c r="AC19" s="33" t="n"/>
-      <x:c r="AD19" s="35" t="str">
+      <x:c r="AB19" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">figures/init-xavier.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC19" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/init-xavier.json. Independent GPU process. grad_p90=0.720357; mean clip fraction=0.000000.</x:v>
+      </x:c>
+      <x:c r="AD19" s="35" t="n">
         <x:f>IF(P19="","",P19-LN(7))</x:f>
-      </x:c>
-      <x:c r="AE19" s="35" t="str">
+        <x:v>0.07626604087982192</x:v>
+      </x:c>
+      <x:c r="AE19" s="35" t="n">
         <x:f>IF(OR(T19="",S19=""),"",T19-S19)</x:f>
-      </x:c>
-      <x:c r="AF19" s="35" t="str">
+        <x:v>0.020018964206283213</x:v>
+      </x:c>
+      <x:c r="AF19" s="35" t="n">
         <x:f>IF(OR(V19="",Seeds!$C$8=""),"",V19-Seeds!$C$8)</x:f>
+        <x:v>-0.002075868733407149</x:v>
       </x:c>
       <x:c r="AG19" s="35" t="str">
         <x:f>IF(OR(AF19="",Seeds!$C$10=""),"",IF(ABS(AF19)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="20" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A20" s="33" t="n"/>
-      <x:c r="B20" s="33" t="n"/>
-      <x:c r="C20" s="33" t="n"/>
-      <x:c r="D20" s="33" t="n"/>
-      <x:c r="E20" s="33" t="n"/>
-      <x:c r="F20" s="33" t="n"/>
-      <x:c r="G20" s="33" t="n"/>
-      <x:c r="H20" s="33" t="n"/>
-      <x:c r="I20" s="33" t="n"/>
-      <x:c r="J20" s="33" t="n"/>
-      <x:c r="K20" s="33" t="n"/>
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A20" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">init-zeros</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">initialization</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">He giữ tín hiệu qua ReLU tốt hơn normal nhỏ; zeros không phá đối xứng và gradient hidden bằng 0.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E20" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F20" s="33" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G20" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="33" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I20" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J20" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">256-128</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K20" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L20" s="33" t="n"/>
-      <x:c r="M20" s="33" t="n"/>
-      <x:c r="N20" s="33" t="n"/>
-      <x:c r="O20" s="33" t="n"/>
-      <x:c r="P20" s="34" t="n"/>
-      <x:c r="Q20" s="34" t="n"/>
-      <x:c r="R20" s="33" t="n"/>
-      <x:c r="S20" s="34" t="n"/>
-      <x:c r="T20" s="34" t="n"/>
-      <x:c r="U20" s="34" t="n"/>
-      <x:c r="V20" s="34" t="n"/>
-      <x:c r="W20" s="33" t="n"/>
-      <x:c r="X20" s="33" t="n"/>
-      <x:c r="Y20" s="33" t="n"/>
+      <x:c r="M20" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">fp32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N20" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">zeros</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O20" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P20" s="34" t="n">
+        <x:v>1.945909990859841</x:v>
+      </x:c>
+      <x:c r="Q20" s="34" t="n">
+        <x:v>1.205200765206818</x:v>
+      </x:c>
+      <x:c r="R20" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="S20" s="34" t="n">
+        <x:v>1.205217598474221</x:v>
+      </x:c>
+      <x:c r="T20" s="34" t="n">
+        <x:v>1.20521924869167</x:v>
+      </x:c>
+      <x:c r="U20" s="34" t="n">
+        <x:v>0.4875970826789441</x:v>
+      </x:c>
+      <x:c r="V20" s="34" t="n">
+        <x:v>0.09364999018625454</x:v>
+      </x:c>
+      <x:c r="W20" s="49" t="n">
+        <x:v>1.318535833500016</x:v>
+      </x:c>
+      <x:c r="X20" s="49" t="n">
+        <x:v>160.59375</x:v>
+      </x:c>
+      <x:c r="Y20" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z20" s="34" t="n"/>
       <x:c r="AA20" s="34" t="n"/>
-      <x:c r="AB20" s="33" t="n"/>
-      <x:c r="AC20" s="33" t="n"/>
-      <x:c r="AD20" s="35" t="str">
+      <x:c r="AB20" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">figures/init-zeros.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC20" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/init-zeros.json. Independent GPU process. grad_p90=0.056345; mean clip fraction=0.000000.</x:v>
+      </x:c>
+      <x:c r="AD20" s="35" t="n">
         <x:f>IF(P20="","",P20-LN(7))</x:f>
-      </x:c>
-      <x:c r="AE20" s="35" t="str">
+        <x:v>-1.5819547227735598e-7</x:v>
+      </x:c>
+      <x:c r="AE20" s="35" t="n">
         <x:f>IF(OR(T20="",S20=""),"",T20-S20)</x:f>
-      </x:c>
-      <x:c r="AF20" s="35" t="str">
+        <x:v>0.000001650217448911917</x:v>
+      </x:c>
+      <x:c r="AF20" s="35" t="n">
         <x:f>IF(OR(V20="",Seeds!$C$8=""),"",V20-Seeds!$C$8)</x:f>
+        <x:v>-0.759860349541994</x:v>
       </x:c>
       <x:c r="AG20" s="35" t="str">
         <x:f>IF(OR(AF20="",Seeds!$C$10=""),"",IF(ABS(AF20)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="21" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A21" s="33" t="n"/>
-      <x:c r="B21" s="33" t="n"/>
-      <x:c r="C21" s="33" t="n"/>
-      <x:c r="D21" s="33" t="n"/>
-      <x:c r="E21" s="33" t="n"/>
-      <x:c r="F21" s="33" t="n"/>
-      <x:c r="G21" s="33" t="n"/>
-      <x:c r="H21" s="33" t="n"/>
-      <x:c r="I21" s="33" t="n"/>
-      <x:c r="J21" s="33" t="n"/>
-      <x:c r="K21" s="33" t="n"/>
+        <x:v>Có</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A21" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">loss-mse</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">loss</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CE phù hợp phân lớp hơn MSE logits/one-hot; chỉ so accuracy/F1, không so trị số loss khác thang.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">mse</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E21" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F21" s="33" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G21" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H21" s="33" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I21" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J21" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">256-128</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K21" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L21" s="33" t="n"/>
-      <x:c r="M21" s="33" t="n"/>
-      <x:c r="N21" s="33" t="n"/>
-      <x:c r="O21" s="33" t="n"/>
-      <x:c r="P21" s="34" t="n"/>
-      <x:c r="Q21" s="34" t="n"/>
-      <x:c r="R21" s="33" t="n"/>
-      <x:c r="S21" s="34" t="n"/>
-      <x:c r="T21" s="34" t="n"/>
-      <x:c r="U21" s="34" t="n"/>
-      <x:c r="V21" s="34" t="n"/>
-      <x:c r="W21" s="33" t="n"/>
-      <x:c r="X21" s="33" t="n"/>
-      <x:c r="Y21" s="33" t="n"/>
+      <x:c r="M21" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">fp32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N21" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">he</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O21" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P21" s="34" t="n">
+        <x:v>0.6358503211013448</x:v>
+      </x:c>
+      <x:c r="Q21" s="34" t="n">
+        <x:v>0.02933052455822363</x:v>
+      </x:c>
+      <x:c r="R21" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="S21" s="34" t="n">
+        <x:v>0.02836624454859914</x:v>
+      </x:c>
+      <x:c r="T21" s="34" t="n">
+        <x:v>0.02933052455822363</x:v>
+      </x:c>
+      <x:c r="U21" s="34" t="n">
+        <x:v>0.8705062283513694</x:v>
+      </x:c>
+      <x:c r="V21" s="34" t="n">
+        <x:v>0.7276654739925651</x:v>
+      </x:c>
+      <x:c r="W21" s="49" t="n">
+        <x:v>1.361007908000005</x:v>
+      </x:c>
+      <x:c r="X21" s="49" t="n">
+        <x:v>160.59716796875</x:v>
+      </x:c>
+      <x:c r="Y21" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z21" s="34" t="n"/>
       <x:c r="AA21" s="34" t="n"/>
-      <x:c r="AB21" s="33" t="n"/>
-      <x:c r="AC21" s="33" t="n"/>
-      <x:c r="AD21" s="35" t="str">
+      <x:c r="AB21" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">figures/loss-mse.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC21" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/loss-mse.json. Independent GPU process. grad_p90=0.114037; mean clip fraction=0.000000.</x:v>
+      </x:c>
+      <x:c r="AD21" s="35" t="n">
         <x:f>IF(P21="","",P21-LN(7))</x:f>
-      </x:c>
-      <x:c r="AE21" s="35" t="str">
+        <x:v>-1.3100598279539684</x:v>
+      </x:c>
+      <x:c r="AE21" s="35" t="n">
         <x:f>IF(OR(T21="",S21=""),"",T21-S21)</x:f>
-      </x:c>
-      <x:c r="AF21" s="35" t="str">
+        <x:v>0.0009642800096244901</x:v>
+      </x:c>
+      <x:c r="AF21" s="35" t="n">
         <x:f>IF(OR(V21="",Seeds!$C$8=""),"",V21-Seeds!$C$8)</x:f>
+        <x:v>-0.12584486573568343</x:v>
       </x:c>
       <x:c r="AG21" s="35" t="str">
         <x:f>IF(OR(AF21="",Seeds!$C$10=""),"",IF(ABS(AF21)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="22" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A22" s="33" t="n"/>
-      <x:c r="B22" s="33" t="n"/>
-      <x:c r="C22" s="33" t="n"/>
-      <x:c r="D22" s="33" t="n"/>
-      <x:c r="E22" s="33" t="n"/>
-      <x:c r="F22" s="33" t="n"/>
-      <x:c r="G22" s="33" t="n"/>
-      <x:c r="H22" s="33" t="n"/>
-      <x:c r="I22" s="33" t="n"/>
-      <x:c r="J22" s="33" t="n"/>
-      <x:c r="K22" s="33" t="n"/>
+        <x:v>Có</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A22" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">precision-bf16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">mixed_precision</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">FP16/BF16 có thể không nhanh hơn với MLP nhỏ; T4 không có BF16 native, nên tốc độ BF16 chỉ là số đo emulation.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E22" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F22" s="33" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G22" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H22" s="33" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I22" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J22" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">256-128</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K22" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L22" s="33" t="n"/>
-      <x:c r="M22" s="33" t="n"/>
-      <x:c r="N22" s="33" t="n"/>
-      <x:c r="O22" s="33" t="n"/>
-      <x:c r="P22" s="34" t="n"/>
-      <x:c r="Q22" s="34" t="n"/>
-      <x:c r="R22" s="33" t="n"/>
-      <x:c r="S22" s="34" t="n"/>
-      <x:c r="T22" s="34" t="n"/>
-      <x:c r="U22" s="34" t="n"/>
-      <x:c r="V22" s="34" t="n"/>
-      <x:c r="W22" s="33" t="n"/>
-      <x:c r="X22" s="33" t="n"/>
-      <x:c r="Y22" s="33" t="n"/>
+      <x:c r="M22" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">bf16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N22" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">he</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O22" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P22" s="34" t="n">
+        <x:v>2.269061788393712</x:v>
+      </x:c>
+      <x:c r="Q22" s="34" t="n">
+        <x:v>0.2367006277546118</x:v>
+      </x:c>
+      <x:c r="R22" s="33" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="S22" s="34" t="n">
+        <x:v>0.2134287808364079</x:v>
+      </x:c>
+      <x:c r="T22" s="34" t="n">
+        <x:v>0.2374560404007484</x:v>
+      </x:c>
+      <x:c r="U22" s="34" t="n">
+        <x:v>0.9055635636066349</x:v>
+      </x:c>
+      <x:c r="V22" s="34" t="n">
+        <x:v>0.8366261256178422</x:v>
+      </x:c>
+      <x:c r="W22" s="49" t="n">
+        <x:v>1.548157692399991</x:v>
+      </x:c>
+      <x:c r="X22" s="49" t="n">
+        <x:v>160.59375</x:v>
+      </x:c>
+      <x:c r="Y22" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z22" s="34" t="n"/>
       <x:c r="AA22" s="34" t="n"/>
-      <x:c r="AB22" s="33" t="n"/>
-      <x:c r="AC22" s="33" t="n"/>
-      <x:c r="AD22" s="35" t="str">
+      <x:c r="AB22" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">figures/precision-bf16.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC22" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/precision-bf16.json. Independent GPU process. grad_p90=0.693962; mean clip fraction=0.000000.</x:v>
+      </x:c>
+      <x:c r="AD22" s="35" t="n">
         <x:f>IF(P22="","",P22-LN(7))</x:f>
-      </x:c>
-      <x:c r="AE22" s="35" t="str">
+        <x:v>0.32315163933839863</x:v>
+      </x:c>
+      <x:c r="AE22" s="35" t="n">
         <x:f>IF(OR(T22="",S22=""),"",T22-S22)</x:f>
-      </x:c>
-      <x:c r="AF22" s="35" t="str">
+        <x:v>0.024027259564340514</x:v>
+      </x:c>
+      <x:c r="AF22" s="35" t="n">
         <x:f>IF(OR(V22="",Seeds!$C$8=""),"",V22-Seeds!$C$8)</x:f>
+        <x:v>-0.016884214110406304</x:v>
       </x:c>
       <x:c r="AG22" s="35" t="str">
         <x:f>IF(OR(AF22="",Seeds!$C$10=""),"",IF(ABS(AF22)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="23" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A23" s="33" t="n"/>
-      <x:c r="B23" s="33" t="n"/>
-      <x:c r="C23" s="33" t="n"/>
-      <x:c r="D23" s="33" t="n"/>
-      <x:c r="E23" s="33" t="n"/>
-      <x:c r="F23" s="33" t="n"/>
-      <x:c r="G23" s="33" t="n"/>
-      <x:c r="H23" s="33" t="n"/>
-      <x:c r="I23" s="33" t="n"/>
-      <x:c r="J23" s="33" t="n"/>
-      <x:c r="K23" s="33" t="n"/>
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" s="20" customFormat="1" ht="36" hidden="0" customHeight="1">
+      <x:c r="A23" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">precision-fp16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">mixed_precision</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">FP16/BF16 có thể không nhanh hơn với MLP nhỏ; T4 không có BF16 native, nên tốc độ BF16 chỉ là số đo emulation.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E23" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F23" s="33" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G23" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" s="33" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I23" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J23" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">256-128</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K23" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L23" s="33" t="n"/>
-      <x:c r="M23" s="33" t="n"/>
-      <x:c r="N23" s="33" t="n"/>
-      <x:c r="O23" s="33" t="n"/>
-      <x:c r="P23" s="34" t="n"/>
-      <x:c r="Q23" s="34" t="n"/>
-      <x:c r="R23" s="33" t="n"/>
-      <x:c r="S23" s="34" t="n"/>
-      <x:c r="T23" s="34" t="n"/>
-      <x:c r="U23" s="34" t="n"/>
-      <x:c r="V23" s="34" t="n"/>
-      <x:c r="W23" s="33" t="n"/>
-      <x:c r="X23" s="33" t="n"/>
-      <x:c r="Y23" s="33" t="n"/>
+      <x:c r="M23" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">fp16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N23" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">he</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O23" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P23" s="34" t="n">
+        <x:v>2.269061788393712</x:v>
+      </x:c>
+      <x:c r="Q23" s="34" t="n">
+        <x:v>0.2359490842181735</x:v>
+      </x:c>
+      <x:c r="R23" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="S23" s="34" t="n">
+        <x:v>0.2123942238831071</x:v>
+      </x:c>
+      <x:c r="T23" s="34" t="n">
+        <x:v>0.2359490842181735</x:v>
+      </x:c>
+      <x:c r="U23" s="34" t="n">
+        <x:v>0.905165551515673</x:v>
+      </x:c>
+      <x:c r="V23" s="34" t="n">
+        <x:v>0.8515042026567495</x:v>
+      </x:c>
+      <x:c r="W23" s="49" t="n">
+        <x:v>1.747236514800011</x:v>
+      </x:c>
+      <x:c r="X23" s="49" t="n">
+        <x:v>160.5947265625</x:v>
+      </x:c>
+      <x:c r="Y23" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z23" s="34" t="n"/>
       <x:c r="AA23" s="34" t="n"/>
-      <x:c r="AB23" s="33" t="n"/>
-      <x:c r="AC23" s="33" t="n"/>
-      <x:c r="AD23" s="35" t="str">
+      <x:c r="AB23" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">figures/precision-fp16.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC23" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/precision-fp16.json. Independent GPU process. grad_p90=0.687714; mean clip fraction=0.000000. AMP gradient overflow; loss finite, GradScaler skips unsafe updates. Missing gradient mean epochs: {"grad_norm":[12,15,19]}.</x:v>
+      </x:c>
+      <x:c r="AD23" s="35" t="n">
         <x:f>IF(P23="","",P23-LN(7))</x:f>
-      </x:c>
-      <x:c r="AE23" s="35" t="str">
+        <x:v>0.32315163933839863</x:v>
+      </x:c>
+      <x:c r="AE23" s="35" t="n">
         <x:f>IF(OR(T23="",S23=""),"",T23-S23)</x:f>
-      </x:c>
-      <x:c r="AF23" s="35" t="str">
+        <x:v>0.023554860335066402</x:v>
+      </x:c>
+      <x:c r="AF23" s="35" t="n">
         <x:f>IF(OR(V23="",Seeds!$C$8=""),"",V23-Seeds!$C$8)</x:f>
+        <x:v>-0.0020061370714989923</x:v>
       </x:c>
       <x:c r="AG23" s="35" t="str">
         <x:f>IF(OR(AF23="",Seeds!$C$10=""),"",IF(ABS(AF23)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="24" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A24" s="33" t="n"/>
-      <x:c r="B24" s="33" t="n"/>
-      <x:c r="C24" s="33" t="n"/>
-      <x:c r="D24" s="33" t="n"/>
-      <x:c r="E24" s="33" t="n"/>
-      <x:c r="F24" s="33" t="n"/>
-      <x:c r="G24" s="33" t="n"/>
-      <x:c r="H24" s="33" t="n"/>
-      <x:c r="I24" s="33" t="n"/>
-      <x:c r="J24" s="33" t="n"/>
-      <x:c r="K24" s="33" t="n"/>
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A24" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgdm-lr0.01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">baseline</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SGD momentum: lr thấp học chậm, lr cao có thể dao động; chọn lr bằng F1 val tại epoch min val loss.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E24" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F24" s="33" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="G24" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="33" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I24" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J24" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">256-128</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K24" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L24" s="33" t="n"/>
-      <x:c r="M24" s="33" t="n"/>
-      <x:c r="N24" s="33" t="n"/>
-      <x:c r="O24" s="33" t="n"/>
-      <x:c r="P24" s="34" t="n"/>
-      <x:c r="Q24" s="34" t="n"/>
-      <x:c r="R24" s="33" t="n"/>
-      <x:c r="S24" s="34" t="n"/>
-      <x:c r="T24" s="34" t="n"/>
-      <x:c r="U24" s="34" t="n"/>
-      <x:c r="V24" s="34" t="n"/>
-      <x:c r="W24" s="33" t="n"/>
-      <x:c r="X24" s="33" t="n"/>
-      <x:c r="Y24" s="33" t="n"/>
+      <x:c r="M24" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">fp32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N24" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">he</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O24" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P24" s="34" t="n">
+        <x:v>2.269061788393712</x:v>
+      </x:c>
+      <x:c r="Q24" s="34" t="n">
+        <x:v>0.3109734395841849</x:v>
+      </x:c>
+      <x:c r="R24" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="S24" s="34" t="n">
+        <x:v>0.2997025162698175</x:v>
+      </x:c>
+      <x:c r="T24" s="34" t="n">
+        <x:v>0.3109734395841849</x:v>
+      </x:c>
+      <x:c r="U24" s="34" t="n">
+        <x:v>0.8746692196811601</x:v>
+      </x:c>
+      <x:c r="V24" s="34" t="n">
+        <x:v>0.7612533557248951</x:v>
+      </x:c>
+      <x:c r="W24" s="49" t="n">
+        <x:v>1.334799609499987</x:v>
+      </x:c>
+      <x:c r="X24" s="49" t="n">
+        <x:v>160.59375</x:v>
+      </x:c>
+      <x:c r="Y24" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z24" s="34" t="n"/>
       <x:c r="AA24" s="34" t="n"/>
-      <x:c r="AB24" s="33" t="n"/>
-      <x:c r="AC24" s="33" t="n"/>
-      <x:c r="AD24" s="35" t="str">
+      <x:c r="AB24" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">figures/sgdm-lr0.01.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC24" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/sgdm-lr0.01.json. Independent GPU process. grad_p90=1.654977; mean clip fraction=0.000000.</x:v>
+      </x:c>
+      <x:c r="AD24" s="35" t="n">
         <x:f>IF(P24="","",P24-LN(7))</x:f>
-      </x:c>
-      <x:c r="AE24" s="35" t="str">
+        <x:v>0.32315163933839863</x:v>
+      </x:c>
+      <x:c r="AE24" s="35" t="n">
         <x:f>IF(OR(T24="",S24=""),"",T24-S24)</x:f>
-      </x:c>
-      <x:c r="AF24" s="35" t="str">
+        <x:v>0.01127092331436741</x:v>
+      </x:c>
+      <x:c r="AF24" s="35" t="n">
         <x:f>IF(OR(V24="",Seeds!$C$8=""),"",V24-Seeds!$C$8)</x:f>
+        <x:v>-0.09225698400335347</x:v>
       </x:c>
       <x:c r="AG24" s="35" t="str">
         <x:f>IF(OR(AF24="",Seeds!$C$10=""),"",IF(ABS(AF24)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="25" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A25" s="33" t="n"/>
-      <x:c r="B25" s="33" t="n"/>
-      <x:c r="C25" s="33" t="n"/>
-      <x:c r="D25" s="33" t="n"/>
-      <x:c r="E25" s="33" t="n"/>
-      <x:c r="F25" s="33" t="n"/>
-      <x:c r="G25" s="33" t="n"/>
-      <x:c r="H25" s="33" t="n"/>
-      <x:c r="I25" s="33" t="n"/>
-      <x:c r="J25" s="33" t="n"/>
-      <x:c r="K25" s="33" t="n"/>
+        <x:v>Có</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A25" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgdm-lr0.05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">baseline</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SGD momentum: lr thấp học chậm, lr cao có thể dao động; chọn lr bằng F1 val tại epoch min val loss.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F25" s="33" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="G25" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H25" s="33" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I25" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J25" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">256-128</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K25" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L25" s="33" t="n"/>
-      <x:c r="M25" s="33" t="n"/>
-      <x:c r="N25" s="33" t="n"/>
-      <x:c r="O25" s="33" t="n"/>
-      <x:c r="P25" s="34" t="n"/>
-      <x:c r="Q25" s="34" t="n"/>
-      <x:c r="R25" s="33" t="n"/>
-      <x:c r="S25" s="34" t="n"/>
-      <x:c r="T25" s="34" t="n"/>
-      <x:c r="U25" s="34" t="n"/>
-      <x:c r="V25" s="34" t="n"/>
-      <x:c r="W25" s="33" t="n"/>
-      <x:c r="X25" s="33" t="n"/>
-      <x:c r="Y25" s="33" t="n"/>
+      <x:c r="M25" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">fp32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N25" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">he</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O25" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P25" s="34" t="n">
+        <x:v>2.269061788393712</x:v>
+      </x:c>
+      <x:c r="Q25" s="34" t="n">
+        <x:v>0.2487494365137099</x:v>
+      </x:c>
+      <x:c r="R25" s="33" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="S25" s="34" t="n">
+        <x:v>0.2328529836482331</x:v>
+      </x:c>
+      <x:c r="T25" s="34" t="n">
+        <x:v>0.2541595102472146</x:v>
+      </x:c>
+      <x:c r="U25" s="34" t="n">
+        <x:v>0.8999591230825499</x:v>
+      </x:c>
+      <x:c r="V25" s="34" t="n">
+        <x:v>0.8351405542256746</x:v>
+      </x:c>
+      <x:c r="W25" s="49" t="n">
+        <x:v>1.341872369199996</x:v>
+      </x:c>
+      <x:c r="X25" s="49" t="n">
+        <x:v>160.59375</x:v>
+      </x:c>
+      <x:c r="Y25" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z25" s="34" t="n"/>
       <x:c r="AA25" s="34" t="n"/>
-      <x:c r="AB25" s="33" t="n"/>
-      <x:c r="AC25" s="33" t="n"/>
-      <x:c r="AD25" s="35" t="str">
+      <x:c r="AB25" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">figures/sgdm-lr0.05.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC25" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/sgdm-lr0.05.json. Independent GPU process. grad_p90=1.019520; mean clip fraction=0.000000.</x:v>
+      </x:c>
+      <x:c r="AD25" s="35" t="n">
         <x:f>IF(P25="","",P25-LN(7))</x:f>
-      </x:c>
-      <x:c r="AE25" s="35" t="str">
+        <x:v>0.32315163933839863</x:v>
+      </x:c>
+      <x:c r="AE25" s="35" t="n">
         <x:f>IF(OR(T25="",S25=""),"",T25-S25)</x:f>
-      </x:c>
-      <x:c r="AF25" s="35" t="str">
+        <x:v>0.021306526598981523</x:v>
+      </x:c>
+      <x:c r="AF25" s="35" t="n">
         <x:f>IF(OR(V25="",Seeds!$C$8=""),"",V25-Seeds!$C$8)</x:f>
+        <x:v>-0.018369785502573954</x:v>
       </x:c>
       <x:c r="AG25" s="35" t="str">
         <x:f>IF(OR(AF25="",Seeds!$C$10=""),"",IF(ABS(AF25)&gt;Seeds!$C$10,"Có","Không"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="26" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A26" s="33" t="n"/>
-      <x:c r="B26" s="33" t="n"/>
-      <x:c r="C26" s="33" t="n"/>
-      <x:c r="D26" s="33" t="n"/>
-      <x:c r="E26" s="33" t="n"/>
-      <x:c r="F26" s="33" t="n"/>
-      <x:c r="G26" s="33" t="n"/>
-      <x:c r="H26" s="33" t="n"/>
-      <x:c r="I26" s="33" t="n"/>
-      <x:c r="J26" s="33" t="n"/>
-      <x:c r="K26" s="33" t="n"/>
+        <x:v>Không</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" s="20" customFormat="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A26" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgdm-lr0.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">baseline</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="47" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SGD momentum: lr thấp học chậm, lr cao có thể dao động; chọn lr bằng F1 val tại epoch min val loss.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E26" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sgd_momentum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F26" s="33" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G26" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H26" s="33" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I26" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J26" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">256-128</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K26" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L26" s="33" t="n"/>
-      <x:c r="M26" s="33" t="n"/>
-      <x:c r="N26" s="33" t="n"/>
-      <x:c r="O26" s="33" t="n"/>
-      <x:c r="P26" s="34" t="n"/>
-      <x:c r="Q26" s="34" t="n"/>
-      <x:c r="R26" s="33" t="n"/>
-      <x:c r="S26" s="34" t="n"/>
-      <x:c r="T26" s="34" t="n"/>
-      <x:c r="U26" s="34" t="n"/>
-      <x:c r="V26" s="34" t="n"/>
-      <x:c r="W26" s="33" t="n"/>
-      <x:c r="X26" s="33" t="n"/>
-      <x:c r="Y26" s="33" t="n"/>
+      <x:c r="M26" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">fp32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N26" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">he</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O26" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P26" s="34" t="n">
+        <x:v>2.269061788393712</x:v>
+      </x:c>
+      <x:c r="Q26" s="34" t="n">
+        <x:v>0.2379235743460702</x:v>
+      </x:c>
+      <x:c r="R26" s="33" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="S26" s="34" t="n">
+        <x:v>0.2208534015460324</x:v>
+      </x:c>
+      <x:c r="T26" s="34" t="n">
+        <x:v>0.2425536006353739</x:v>
+      </x:c>
+      <x:c r="U26" s="34" t="n">
+        <x:v>0.9053806931864633</x:v>
+      </x:c>
+      <x:c r="V26" s="34" t="n">
+        <x:v>0.8390357563558714</x:v>
+      </x:c>
+      <x:c r="W26" s="49" t="n">
+        <x:v>1.34452435555001</x:v>
+      </x:c>
+      <x:c r="X26" s="49" t="n">
+        <x:v>160.59375</x:v>
+      </x:c>
+      <x:c r="Y26" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z26" s="34" t="n"/>
       <x:c r="AA26" s="34" t="n"/>
-      <x:c r="AB26" s="33" t="n"/>
-      <x:c r="AC26" s="33" t="n"/>
-      <x:c r="AD26" s="35" t="str">
+      <x:c r="AB26" s="33" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">figures/sgdm-lr0.1.png</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="AC26" s="47" t="str">
+        <x:v>Prediction recorded before worker in planned/sgdm-lr0.1.json. Independent GPU process. grad_p90=0.696241; mean clip fraction=0.000000.</x:v>
+      </x:c>
+      <x:c r="AD26" s="35" t="n">
         <x:f>IF(P26="","",P26-LN(7))</x:f>
-      </x:c>
-      <x:c r="AE26" s="35" t="str">
+        <x:v>0.32315163933839863</x:v>
+      </x:c>
+      <x:c r="AE26" s="35" t="n">
         <x:f>IF(OR(T26="",S26=""),"",T26-S26)</x:f>
-      </x:c>
-      <x:c r="AF26" s="35" t="str">
+        <x:v>0.02170019908934151</x:v>
+      </x:c>
+      <x:c r="AF26" s="35" t="n">
         <x:f>IF(OR(V26="",Seeds!$C$8=""),"",V26-Seeds!$C$8)</x:f>
+        <x:v>-0.01447458337237717</x:v>
       </x:c>
       <x:c r="AG26" s="35" t="str">
         <x:f>IF(OR(AF26="",Seeds!$C$10=""),"",IF(ABS(AF26)&gt;Seeds!$C$10,"Có","Không"))</x:f>
+        <x:v>Không</x:v>
       </x:c>
     </x:row>
     <x:row r="27" s="20" customFormat="1" ht="15" customHeight="1">
@@ -5415,15 +6089,15 @@
       </x:c>
       <x:c r="B2" s="35" t="n">
         <x:f>IF($A2="","",IFERROR(IF(INDEX(Experiments!$U$2:$U$61,MATCH($A2,Experiments!$A$2:$A$61,0))="","",INDEX(Experiments!$U$2:$U$61,MATCH($A2,Experiments!$A$2:$A$61,0))),""))</x:f>
-        <x:v>0.8839310686086788</x:v>
+        <x:v>0.9053806931864633</x:v>
       </x:c>
       <x:c r="C2" s="35" t="n">
         <x:f>IF($A2="","",IFERROR(IF(INDEX(Experiments!$V$2:$V$61,MATCH($A2,Experiments!$A$2:$A$61,0))="","",INDEX(Experiments!$V$2:$V$61,MATCH($A2,Experiments!$A$2:$A$61,0))),""))</x:f>
-        <x:v>0.8105385838093785</x:v>
+        <x:v>0.8390357563558714</x:v>
       </x:c>
       <x:c r="D2" s="35" t="n">
         <x:f>IF($A2="","",IFERROR(IF(INDEX(Experiments!$Q$2:$Q$61,MATCH($A2,Experiments!$A$2:$A$61,0))="","",INDEX(Experiments!$Q$2:$Q$61,MATCH($A2,Experiments!$A$2:$A$61,0))),""))</x:f>
-        <x:v>0.287590792568889</x:v>
+        <x:v>0.2379235743460702</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="20" customFormat="1" ht="15" customHeight="1">
@@ -5434,15 +6108,15 @@
       </x:c>
       <x:c r="B3" s="35" t="n">
         <x:f>IF($A3="","",IFERROR(IF(INDEX(Experiments!$U$2:$U$61,MATCH($A3,Experiments!$A$2:$A$61,0))="","",INDEX(Experiments!$U$2:$U$61,MATCH($A3,Experiments!$A$2:$A$61,0))),""))</x:f>
-        <x:v>0.884587250704589</x:v>
+        <x:v>0.909984724941374</x:v>
       </x:c>
       <x:c r="C3" s="35" t="n">
         <x:f>IF($A3="","",IFERROR(IF(INDEX(Experiments!$V$2:$V$61,MATCH($A3,Experiments!$A$2:$A$61,0))="","",INDEX(Experiments!$V$2:$V$61,MATCH($A3,Experiments!$A$2:$A$61,0))),""))</x:f>
-        <x:v>0.8128493532287756</x:v>
+        <x:v>0.860050003346835</x:v>
       </x:c>
       <x:c r="D3" s="35" t="n">
         <x:f>IF($A3="","",IFERROR(IF(INDEX(Experiments!$Q$2:$Q$61,MATCH($A3,Experiments!$A$2:$A$61,0))="","",INDEX(Experiments!$Q$2:$Q$61,MATCH($A3,Experiments!$A$2:$A$61,0))),""))</x:f>
-        <x:v>0.2875723438817323</x:v>
+        <x:v>0.2278535272960154</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="20" customFormat="1" ht="15" customHeight="1">
@@ -5453,15 +6127,15 @@
       </x:c>
       <x:c r="B4" s="35" t="n">
         <x:f>IF($A4="","",IFERROR(IF(INDEX(Experiments!$U$2:$U$61,MATCH($A4,Experiments!$A$2:$A$61,0))="","",INDEX(Experiments!$U$2:$U$61,MATCH($A4,Experiments!$A$2:$A$61,0))),""))</x:f>
-        <x:v>0.8803489597900217</x:v>
+        <x:v>0.9091026440911341</x:v>
       </x:c>
       <x:c r="C4" s="35" t="n">
         <x:f>IF($A4="","",IFERROR(IF(INDEX(Experiments!$V$2:$V$61,MATCH($A4,Experiments!$A$2:$A$61,0))="","",INDEX(Experiments!$V$2:$V$61,MATCH($A4,Experiments!$A$2:$A$61,0))),""))</x:f>
-        <x:v>0.8083332183474771</x:v>
+        <x:v>0.861445259482039</x:v>
       </x:c>
       <x:c r="D4" s="35" t="n">
         <x:f>IF($A4="","",IFERROR(IF(INDEX(Experiments!$Q$2:$Q$61,MATCH($A4,Experiments!$A$2:$A$61,0))="","",INDEX(Experiments!$Q$2:$Q$61,MATCH($A4,Experiments!$A$2:$A$61,0))),""))</x:f>
-        <x:v>0.2934093584084592</x:v>
+        <x:v>0.2276589681332745</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="20" customFormat="1" ht="15" customHeight="1">
@@ -5496,15 +6170,15 @@
       </x:c>
       <x:c r="B8" s="35" t="n">
         <x:f>IF(COUNT(B2:B6)=0,"",AVERAGE(B2:B6))</x:f>
-        <x:v>0.8829557597010965</x:v>
+        <x:v>0.9081560207396571</x:v>
       </x:c>
       <x:c r="C8" s="35" t="n">
         <x:f>IF(COUNT(C2:C6)=0,"",AVERAGE(C2:C6))</x:f>
-        <x:v>0.810573718461877</x:v>
+        <x:v>0.8535103397282485</x:v>
       </x:c>
       <x:c r="D8" s="35" t="n">
         <x:f>IF(COUNT(D2:D6)=0,"",AVERAGE(D2:D6))</x:f>
-        <x:v>0.28952416495302685</x:v>
+        <x:v>0.2311453565917867</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="20" customFormat="1" ht="15" customHeight="1">
@@ -5515,15 +6189,15 @@
       </x:c>
       <x:c r="B9" s="35" t="n">
         <x:f>IF(COUNT(B2:B6)&lt;2,"",STDEV(B2:B6))</x:f>
-        <x:v>0.0022812711517995635</x:v>
+        <x:v>0.002443634368564064</x:v>
       </x:c>
       <x:c r="C9" s="35" t="n">
         <x:f>IF(COUNT(C2:C6)&lt;2,"",STDEV(C2:C6))</x:f>
-        <x:v>0.0022582724369249584</x:v>
+        <x:v>0.012554754389219557</x:v>
       </x:c>
       <x:c r="D9" s="35" t="n">
         <x:f>IF(COUNT(D2:D6)&lt;2,"",STDEV(D2:D6))</x:f>
-        <x:v>0.003364688875381412</x:v>
+        <x:v>0.005870914772019319</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="20" customFormat="1" ht="15" customHeight="1">
@@ -5534,15 +6208,15 @@
       </x:c>
       <x:c r="B10" s="35" t="n">
         <x:f>IF(B9="","",2*B9)</x:f>
-        <x:v>0.004562542303599127</x:v>
+        <x:v>0.004887268737128128</x:v>
       </x:c>
       <x:c r="C10" s="35" t="n">
         <x:f>IF(C9="","",2*C9)</x:f>
-        <x:v>0.004516544873849917</x:v>
+        <x:v>0.025109508778439114</x:v>
       </x:c>
       <x:c r="D10" s="35" t="n">
         <x:f>IF(D9="","",2*D9)</x:f>
-        <x:v>0.006729377750762824</x:v>
+        <x:v>0.011741829544038638</x:v>
       </x:c>
     </x:row>
     <x:row r="12" s="20" customFormat="1" ht="15" customHeight="1">
@@ -5568,12 +6242,15 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" style="19" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10" style="19" customWidth="1"/>
+    <x:col min="1" max="1" width="35" style="19" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="36" style="19" hidden="0" customWidth="1"/>
     <x:col min="3" max="5" width="16" style="19" customWidth="1"/>
-    <x:col min="6" max="6" width="14" style="19" customWidth="1"/>
+    <x:col min="6" max="6" width="18" style="19" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="16" style="19" customWidth="1"/>
-    <x:col min="8" max="8" width="50" style="19" customWidth="1"/>
+    <x:col min="8" max="8" width="62" style="19" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="20" customFormat="1" ht="31.5" customHeight="1">
@@ -5626,23 +6303,23 @@
       </x:c>
       <x:c r="B2" s="37" t="n">
         <x:f>COUNTIF(Experiments!$B$2:$B$61,A2)</x:f>
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C2" s="37" t="n">
         <x:f>COUNTIFS(Experiments!$B$2:$B$61,A2,Experiments!$V$2:$V$61,"&lt;&gt;")</x:f>
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D2" s="35" t="n">
         <x:f>IF(C2=0,"",_xlfn.MAXIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A2))</x:f>
-        <x:v>0.8128493532287756</x:v>
+        <x:v>0.861445259482039</x:v>
       </x:c>
       <x:c r="E2" s="35" t="n">
         <x:f>IF(C2=0,"",_xlfn.MINIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A2))</x:f>
-        <x:v>0.8083332183474771</x:v>
+        <x:v>0.761253355724895</x:v>
       </x:c>
       <x:c r="F2" s="35" t="n">
         <x:f>IF(C2=0,"",_xlfn.MAXIFS(Experiments!$U$2:$U$61,Experiments!$B$2:$B$61,A2))</x:f>
-        <x:v>0.884587250704589</x:v>
+        <x:v>0.909984724941374</x:v>
       </x:c>
       <x:c r="G2" s="37" t="inlineStr">
         <x:is>
@@ -5650,7 +6327,7 @@
         </x:is>
       </x:c>
       <x:c r="H2" s="39" t="str">
-        <x:v>3 seed baseline; ngưỡng nhiễu trong Seeds.</x:v>
+        <x:v>SGD momentum 0.9, batch512; lr chọn qua val; 3 seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
@@ -5669,22 +6346,22 @@
       </x:c>
       <x:c r="D3" s="35" t="n">
         <x:f>IF(C3=0,"",_xlfn.MAXIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A3))</x:f>
-        <x:v>0.7590204129234761</x:v>
+        <x:v>0.7276654739925651</x:v>
       </x:c>
       <x:c r="E3" s="35" t="n">
         <x:f>IF(C3=0,"",_xlfn.MINIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A3))</x:f>
-        <x:v>0.7590204129234761</x:v>
+        <x:v>0.7276654739925651</x:v>
       </x:c>
       <x:c r="F3" s="35" t="n">
         <x:f>IF(C3=0,"",_xlfn.MAXIFS(Experiments!$U$2:$U$61,Experiments!$B$2:$B$61,A3))</x:f>
-        <x:v>0.8743465071749748</x:v>
+        <x:v>0.8705062283513694</x:v>
       </x:c>
       <x:c r="G3" s="37" t="str">
         <x:f>IF(C3&gt;0,"Có","Chưa")</x:f>
         <x:v>Có</x:v>
       </x:c>
       <x:c r="H3" s="39" t="str">
-        <x:v>MSE logits kém CE về macro-F1.</x:v>
+        <x:v>loss-mse: F1=0.727665; Δbaseline=-0.111370. Một seed mỗi thử nghiệm.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
@@ -5695,35 +6372,37 @@
       </x:c>
       <x:c r="B4" s="37" t="n">
         <x:f>COUNTIF(Experiments!$B$2:$B$61,A4)</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C4" s="37" t="n">
         <x:f>COUNTIFS(Experiments!$B$2:$B$61,A4,Experiments!$V$2:$V$61,"&lt;&gt;")</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D4" s="35" t="n">
         <x:f>IF(C4=0,"",_xlfn.MAXIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A4))</x:f>
-        <x:v>0.8105385838093785</x:v>
+        <x:v>0.8677466182111557</x:v>
       </x:c>
       <x:c r="E4" s="35" t="n">
         <x:f>IF(C4=0,"",_xlfn.MINIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A4))</x:f>
-        <x:v>0.6616020830040074</x:v>
+        <x:v>0.7877390598660482</x:v>
       </x:c>
       <x:c r="F4" s="35" t="n">
         <x:f>IF(C4=0,"",_xlfn.MAXIFS(Experiments!$U$2:$U$61,Experiments!$B$2:$B$61,A4))</x:f>
-        <x:v>0.8839310686086788</x:v>
+        <x:v>0.9152879671263527</x:v>
       </x:c>
       <x:c r="G4" s="37" t="str">
         <x:f>IF(C4&gt;0,"Có","Chưa")</x:f>
         <x:v>Có</x:v>
       </x:c>
       <x:c r="H4" s="39" t="str">
-        <x:v>Adam lr=0.001 tốt nhất trong lưới đã thử.</x:v>
+        <x:v>adam-lr0.003: F1=0.867747; Δbaseline=0.028711. Một seed mỗi thử nghiệm.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="31" t="str">
-        <x:v>hyperparameter</x:v>
+      <x:c r="A5" s="31" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">hyperparameter</x:t>
+        </x:is>
       </x:c>
       <x:c r="B5" s="37" t="n">
         <x:f>COUNTIF(Experiments!$B$2:$B$61,A5)</x:f>
@@ -5735,22 +6414,22 @@
       </x:c>
       <x:c r="D5" s="35" t="n">
         <x:f>IF(C5=0,"",_xlfn.MAXIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A5))</x:f>
-        <x:v>0.7347919884872669</x:v>
+        <x:v>0.7969625312167096</x:v>
       </x:c>
       <x:c r="E5" s="35" t="n">
         <x:f>IF(C5=0,"",_xlfn.MINIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A5))</x:f>
-        <x:v>0.7347919884872669</x:v>
+        <x:v>0.7969625312167096</x:v>
       </x:c>
       <x:c r="F5" s="35" t="n">
         <x:f>IF(C5=0,"",_xlfn.MAXIFS(Experiments!$U$2:$U$61,Experiments!$B$2:$B$61,A5))</x:f>
-        <x:v>0.8458402357952712</x:v>
+        <x:v>0.8851788902992621</x:v>
       </x:c>
       <x:c r="G5" s="37" t="str">
         <x:f>IF(C5&gt;0,"Có","Chưa")</x:f>
         <x:v>Có</x:v>
       </x:c>
       <x:c r="H5" s="39" t="str">
-        <x:v>lr=0.0003 hội tụ chậm hơn lr=0.001.</x:v>
+        <x:v>batch2048: F1=0.796963; Δbaseline=-0.042073. Một seed mỗi thử nghiệm.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
@@ -5769,22 +6448,22 @@
       </x:c>
       <x:c r="D6" s="35" t="n">
         <x:f>IF(C6=0,"",_xlfn.MAXIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A6))</x:f>
-        <x:v>0.7495524199248325</x:v>
+        <x:v>0.7874882114860531</x:v>
       </x:c>
       <x:c r="E6" s="35" t="n">
         <x:f>IF(C6=0,"",_xlfn.MINIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A6))</x:f>
-        <x:v>0.7495524199248325</x:v>
+        <x:v>0.7874882114860531</x:v>
       </x:c>
       <x:c r="F6" s="35" t="n">
         <x:f>IF(C6=0,"",_xlfn.MAXIFS(Experiments!$U$2:$U$61,Experiments!$B$2:$B$61,A6))</x:f>
-        <x:v>0.8495944579505604</x:v>
+        <x:v>0.8727867300617457</x:v>
       </x:c>
       <x:c r="G6" s="37" t="str">
         <x:f>IF(C6&gt;0,"Có","Chưa")</x:f>
         <x:v>Có</x:v>
       </x:c>
       <x:c r="H6" s="39" t="str">
-        <x:v>Dropout 0.3 làm giảm macro-F1.</x:v>
+        <x:v>dropout-p03: F1=0.787488; Δbaseline=-0.051548. Một seed mỗi thử nghiệm.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
@@ -5795,35 +6474,37 @@
       </x:c>
       <x:c r="B7" s="37" t="n">
         <x:f>COUNTIF(Experiments!$B$2:$B$61,A7)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C7" s="37" t="n">
         <x:f>COUNTIFS(Experiments!$B$2:$B$61,A7,Experiments!$V$2:$V$61,"&lt;&gt;")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D7" s="35" t="n">
         <x:f>IF(C7=0,"",_xlfn.MAXIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A7))</x:f>
-        <x:v>0.8676104419728523</x:v>
+        <x:v>0.8441129852605526</x:v>
       </x:c>
       <x:c r="E7" s="35" t="n">
         <x:f>IF(C7=0,"",_xlfn.MINIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A7))</x:f>
-        <x:v>0.8671875241333343</x:v>
+        <x:v>0.7731754847049565</x:v>
       </x:c>
       <x:c r="F7" s="35" t="n">
         <x:f>IF(C7=0,"",_xlfn.MAXIFS(Experiments!$U$2:$U$61,Experiments!$B$2:$B$61,A7))</x:f>
-        <x:v>0.9107592349562187</x:v>
+        <x:v>0.9026914223015856</x:v>
       </x:c>
       <x:c r="G7" s="37" t="str">
         <x:f>IF(C7&gt;0,"Có","Chưa")</x:f>
         <x:v>Có</x:v>
       </x:c>
       <x:c r="H7" s="39" t="str">
-        <x:v>lr=0.01 có/không clip đều hội tụ.</x:v>
+        <x:v>clip-normal: F1=0.844113; Δbaseline=0.005077. Một seed mỗi thử nghiệm.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="31" t="str">
-        <x:v>mixed_precision</x:v>
+      <x:c r="A8" s="31" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">mixed_precision</x:t>
+        </x:is>
       </x:c>
       <x:c r="B8" s="37" t="n">
         <x:f>COUNTIF(Experiments!$B$2:$B$61,A8)</x:f>
@@ -5835,54 +6516,56 @@
       </x:c>
       <x:c r="D8" s="35" t="n">
         <x:f>IF(C8=0,"",_xlfn.MAXIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A8))</x:f>
-        <x:v>0.8127790715003889</x:v>
+        <x:v>0.8515042026567495</x:v>
       </x:c>
       <x:c r="E8" s="35" t="n">
         <x:f>IF(C8=0,"",_xlfn.MINIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A8))</x:f>
-        <x:v>0.8121172525672452</x:v>
+        <x:v>0.8366261256178422</x:v>
       </x:c>
       <x:c r="F8" s="35" t="n">
         <x:f>IF(C8=0,"",_xlfn.MAXIFS(Experiments!$U$2:$U$61,Experiments!$B$2:$B$61,A8))</x:f>
-        <x:v>0.8846948215399841</x:v>
+        <x:v>0.9055635636066349</x:v>
       </x:c>
       <x:c r="G8" s="37" t="str">
         <x:f>IF(C8&gt;0,"Có","Chưa")</x:f>
         <x:v>Có</x:v>
       </x:c>
       <x:c r="H8" s="39" t="str">
-        <x:v>FP16/BF16 không nhanh hơn FP32 ở mạng này.</x:v>
+        <x:v>precision-fp16: F1=0.851504; Δbaseline=0.012468. Một seed mỗi thử nghiệm.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="20" customFormat="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="31" t="str">
-        <x:v>initialization</x:v>
+      <x:c r="A9" s="31" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">initialization</x:t>
+        </x:is>
       </x:c>
       <x:c r="B9" s="37" t="n">
         <x:f>COUNTIF(Experiments!$B$2:$B$61,A9)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C9" s="37" t="n">
         <x:f>COUNTIFS(Experiments!$B$2:$B$61,A9,Experiments!$V$2:$V$61,"&lt;&gt;")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D9" s="35" t="n">
         <x:f>IF(C9=0,"",_xlfn.MAXIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A9))</x:f>
-        <x:v>0.8038252517683885</x:v>
+        <x:v>0.8514344709948414</x:v>
       </x:c>
       <x:c r="E9" s="35" t="n">
         <x:f>IF(C9=0,"",_xlfn.MINIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A9))</x:f>
-        <x:v>0.7561769579452472</x:v>
+        <x:v>0.09364999018625454</x:v>
       </x:c>
       <x:c r="F9" s="35" t="n">
         <x:f>IF(C9=0,"",_xlfn.MAXIFS(Experiments!$U$2:$U$61,Experiments!$B$2:$B$61,A9))</x:f>
-        <x:v>0.8782835997504357</x:v>
+        <x:v>0.9072309115552591</x:v>
       </x:c>
       <x:c r="G9" s="37" t="str">
         <x:f>IF(C9&gt;0,"Có","Chưa")</x:f>
         <x:v>Có</x:v>
       </x:c>
       <x:c r="H9" s="39" t="str">
-        <x:v>He tốt nhất trong các khởi tạo đã thử.</x:v>
+        <x:v>init-xavier: F1=0.851434; Δbaseline=0.012399. Một seed mỗi thử nghiệm.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="20" customFormat="1" ht="15" customHeight="1">
@@ -5923,20 +6606,23 @@
       </x:c>
       <x:c r="B11" s="37" t="n">
         <x:f>COUNTIF(Experiments!$B$2:$B$61,A11)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C11" s="37" t="n">
         <x:f>COUNTIFS(Experiments!$B$2:$B$61,A11,Experiments!$V$2:$V$61,"&lt;&gt;")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D11" s="35" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D11" s="35" t="n">
         <x:f>IF(C11=0,"",_xlfn.MAXIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A11))</x:f>
-      </x:c>
-      <x:c r="E11" s="35" t="str">
+        <x:v>0.8718252825287924</x:v>
+      </x:c>
+      <x:c r="E11" s="35" t="n">
         <x:f>IF(C11=0,"",_xlfn.MINIFS(Experiments!$V$2:$V$61,Experiments!$B$2:$B$61,A11))</x:f>
-      </x:c>
-      <x:c r="F11" s="35" t="str">
+        <x:v>0.86256369796698</x:v>
+      </x:c>
+      <x:c r="F11" s="35" t="n">
         <x:f>IF(C11=0,"",_xlfn.MAXIFS(Experiments!$U$2:$U$61,Experiments!$B$2:$B$61,A11))</x:f>
+        <x:v>0.9172242421634647</x:v>
       </x:c>
       <x:c r="G11" s="37" t="inlineStr">
         <x:is>
@@ -5957,8 +6643,856 @@
       </x:c>
     </x:row>
     <x:row r="14" s="20" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A14" s="22" t="str">
-        <x:v>7 chủ đề: loss, optimizer, hyperparameter, dropout, clipping, mixed_precision, initialization.</x:v>
+      <x:c r="A14" s="22" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">7 chủ đề: loss, optimizer, hyperparameter, dropout, clipping, mixed_precision, initialization.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="45" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Metric</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="45" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">exp_id / source</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">value</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">std / detail</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E20" s="46"/>
+      <x:c r="F20" s="46"/>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Baseline val macro-F1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1..3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="42" t="n">
+        <x:v>0.8535103397282485</x:v>
+      </x:c>
+      <x:c r="D21" s="42" t="n">
+        <x:v>0.01255475438921956</x:v>
+      </x:c>
+      <x:c r="E21" s="42"/>
+      <x:c r="F21" s="42"/>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Baseline val accuracy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1..3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="42" t="n">
+        <x:v>0.9081560207396571</x:v>
+      </x:c>
+      <x:c r="D22" s="42" t="n">
+        <x:v>0.002443634368564064</x:v>
+      </x:c>
+      <x:c r="E22" s="42"/>
+      <x:c r="F22" s="42"/>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Final eval macro-F1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003; final-s2; final-s3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="42" t="n">
+        <x:v>0.8688705339962425</x:v>
+      </x:c>
+      <x:c r="D23" s="42" t="n">
+        <x:v>0.003280089587279769</x:v>
+      </x:c>
+      <x:c r="E23" s="42"/>
+      <x:c r="F23" s="42"/>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Noise threshold 2 sigma</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1..3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="42" t="n">
+        <x:v>0.02510950877843911</x:v>
+      </x:c>
+      <x:c r="D24" s="42" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Validation only</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E24" s="42"/>
+      <x:c r="F24" s="42"/>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Overfit20 final loss</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1 health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="42" t="n">
+        <x:v>4.392843038658611e-06</x:v>
+      </x:c>
+      <x:c r="D25" s="42" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">500 Adam updates, lr=.01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="42"/>
+      <x:c r="F25" s="42"/>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Overfit20 accuracy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1 health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="42" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D26" s="42" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">20 samples</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E26" s="42"/>
+      <x:c r="F26" s="42"/>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Majority val accuracy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1 health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="42" t="n">
+        <x:v>0.4875970780849457</x:v>
+      </x:c>
+      <x:c r="D27" s="42" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Fixed stratified split</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E27" s="42"/>
+      <x:c r="F27" s="42"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Uniform logits CE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B28" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1 health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" s="42" t="n">
+        <x:v>1.945909976959229</x:v>
+      </x:c>
+      <x:c r="D28" s="42" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ln(7)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E28" s="42"/>
+      <x:c r="F28" s="42"/>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Recorded epoch seconds</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B29" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">all experiment rows</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" s="42" t="n">
+        <x:v>685.4039501519983</x:v>
+      </x:c>
+      <x:c r="D29" s="42" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Excludes setup, plotting, health, scoring</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E29" s="42"/>
+      <x:c r="F29" s="42"/>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Final minus baseline eval F1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B30" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" s="42" t="n">
+        <x:v>0.02900697774102767</x:v>
+      </x:c>
+      <x:c r="D30" s="42" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Baseline eval has one seed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E30" s="42"/>
+      <x:c r="F30" s="42"/>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Final val/eval F1 gap</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B31" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31" s="42" t="n">
+        <x:v>0.002252563336577751</x:v>
+      </x:c>
+      <x:c r="D31" s="42" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">eval minus val</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E31" s="42"/>
+      <x:c r="F31" s="42"/>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Init he std after ReLU1/2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B32" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1 health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" s="42" t="n">
+        <x:v>0.3904455602169037</x:v>
+      </x:c>
+      <x:c r="D32" s="42" t="n">
+        <x:v>0.3660891950130463</x:v>
+      </x:c>
+      <x:c r="E32" s="42"/>
+      <x:c r="F32" s="42"/>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Init xavier std after ReLU1/2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B33" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1 health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" s="42" t="n">
+        <x:v>0.1629583239555359</x:v>
+      </x:c>
+      <x:c r="D33" s="42" t="n">
+        <x:v>0.1247548162937164</x:v>
+      </x:c>
+      <x:c r="E33" s="42"/>
+      <x:c r="F33" s="42"/>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Init normal std after ReLU1/2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B34" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1 health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="42" t="n">
+        <x:v>0.02028814703226089</x:v>
+      </x:c>
+      <x:c r="D34" s="42" t="n">
+        <x:v>0.002152156084775925</x:v>
+      </x:c>
+      <x:c r="E34" s="42"/>
+      <x:c r="F34" s="42"/>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="A35" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Init zeros std after ReLU1/2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B35" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1 health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" s="42" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D35" s="42" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="42"/>
+      <x:c r="F35" s="42"/>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="45" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Per-class eval: base-s1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B36" s="45" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">class</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">support</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D36" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">precision</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E36" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">recall</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F36" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F1</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B37" s="41" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C37" s="42" t="n">
+        <x:v>42368</x:v>
+      </x:c>
+      <x:c r="D37" s="42" t="n">
+        <x:v>0.9015601432880844</x:v>
+      </x:c>
+      <x:c r="E37" s="42" t="n">
+        <x:v>0.9029220166163142</x:v>
+      </x:c>
+      <x:c r="F37" s="42" t="n">
+        <x:v>0.9022405660377357</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B38" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C38" s="42" t="n">
+        <x:v>56661</x:v>
+      </x:c>
+      <x:c r="D38" s="42" t="n">
+        <x:v>0.9092774970247849</x:v>
+      </x:c>
+      <x:c r="E38" s="42" t="n">
+        <x:v>0.9304283369513422</x:v>
+      </x:c>
+      <x:c r="F38" s="42" t="n">
+        <x:v>0.9197313328681088</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B39" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C39" s="42" t="n">
+        <x:v>7151</x:v>
+      </x:c>
+      <x:c r="D39" s="42" t="n">
+        <x:v>0.8972320794889993</x:v>
+      </x:c>
+      <x:c r="E39" s="42" t="n">
+        <x:v>0.8839323171584393</x:v>
+      </x:c>
+      <x:c r="F39" s="42" t="n">
+        <x:v>0.8905325443786982</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B40" s="41" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C40" s="42" t="n">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="D40" s="42" t="n">
+        <x:v>0.7618213660245184</x:v>
+      </x:c>
+      <x:c r="E40" s="42" t="n">
+        <x:v>0.7923497267759563</x:v>
+      </x:c>
+      <x:c r="F40" s="42" t="n">
+        <x:v>0.7767857142857144</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="A41" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B41" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C41" s="42" t="n">
+        <x:v>1899</x:v>
+      </x:c>
+      <x:c r="D41" s="42" t="n">
+        <x:v>0.8161073825503355</x:v>
+      </x:c>
+      <x:c r="E41" s="42" t="n">
+        <x:v>0.640337019483939</x:v>
+      </x:c>
+      <x:c r="F41" s="42" t="n">
+        <x:v>0.7176158158748894</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B42" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C42" s="42" t="n">
+        <x:v>3473</x:v>
+      </x:c>
+      <x:c r="D42" s="42" t="n">
+        <x:v>0.8488992661774516</x:v>
+      </x:c>
+      <x:c r="E42" s="42" t="n">
+        <x:v>0.7327958537287648</x:v>
+      </x:c>
+      <x:c r="F42" s="42" t="n">
+        <x:v>0.7865863081440272</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">base-s1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B43" s="41" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C43" s="42" t="n">
+        <x:v>4102</x:v>
+      </x:c>
+      <x:c r="D43" s="42" t="n">
+        <x:v>0.9436008676789588</x:v>
+      </x:c>
+      <x:c r="E43" s="42" t="n">
+        <x:v>0.8483666504144319</x:v>
+      </x:c>
+      <x:c r="F43" s="42" t="n">
+        <x:v>0.8934531450577664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="45" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Per-class eval: adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B44" s="45" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">class</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C44" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">support</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D44" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">precision</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E44" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">recall</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F44" s="46" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F1</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B45" s="41" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C45" s="42" t="n">
+        <x:v>42368</x:v>
+      </x:c>
+      <x:c r="D45" s="42" t="n">
+        <x:v>0.9283215921966599</x:v>
+      </x:c>
+      <x:c r="E45" s="42" t="n">
+        <x:v>0.8895392749244713</x:v>
+      </x:c>
+      <x:c r="F45" s="42" t="n">
+        <x:v>0.9085167417978448</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B46" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C46" s="42" t="n">
+        <x:v>56661</x:v>
+      </x:c>
+      <x:c r="D46" s="42" t="n">
+        <x:v>0.9118872319804119</x:v>
+      </x:c>
+      <x:c r="E46" s="42" t="n">
+        <x:v>0.9464887665237112</x:v>
+      </x:c>
+      <x:c r="F46" s="42" t="n">
+        <x:v>0.9288658722460857</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B47" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C47" s="42" t="n">
+        <x:v>7151</x:v>
+      </x:c>
+      <x:c r="D47" s="42" t="n">
+        <x:v>0.9300295857988166</x:v>
+      </x:c>
+      <x:c r="E47" s="42" t="n">
+        <x:v>0.8791777373793875</x:v>
+      </x:c>
+      <x:c r="F47" s="42" t="n">
+        <x:v>0.9038890086981526</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B48" s="41" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C48" s="42" t="n">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="D48" s="42" t="n">
+        <x:v>0.7149059334298119</x:v>
+      </x:c>
+      <x:c r="E48" s="42" t="n">
+        <x:v>0.8998178506375227</x:v>
+      </x:c>
+      <x:c r="F48" s="42" t="n">
+        <x:v>0.7967741935483871</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B49" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C49" s="42" t="n">
+        <x:v>1899</x:v>
+      </x:c>
+      <x:c r="D49" s="42" t="n">
+        <x:v>0.8296795952782462</x:v>
+      </x:c>
+      <x:c r="E49" s="42" t="n">
+        <x:v>0.7772511848341233</x:v>
+      </x:c>
+      <x:c r="F49" s="42" t="n">
+        <x:v>0.8026101141924958</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B50" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C50" s="42" t="n">
+        <x:v>3473</x:v>
+      </x:c>
+      <x:c r="D50" s="42" t="n">
+        <x:v>0.8078282141886383</x:v>
+      </x:c>
+      <x:c r="E50" s="42" t="n">
+        <x:v>0.8557443132738267</x:v>
+      </x:c>
+      <x:c r="F50" s="42" t="n">
+        <x:v>0.831096196868009</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="41" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">adam-lr0.003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B51" s="41" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C51" s="42" t="n">
+        <x:v>4102</x:v>
+      </x:c>
+      <x:c r="D51" s="42" t="n">
+        <x:v>0.9438867438867439</x:v>
+      </x:c>
+      <x:c r="E51" s="42" t="n">
+        <x:v>0.893954168698196</x:v>
+      </x:c>
+      <x:c r="F51" s="42" t="n">
+        <x:v>0.9182421434831601</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="41"/>
+      <x:c r="B52" s="41"/>
+      <x:c r="C52" s="42"/>
+      <x:c r="D52" s="42"/>
+      <x:c r="E52" s="42"/>
+      <x:c r="F52" s="42"/>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="41"/>
+      <x:c r="B53" s="41"/>
+      <x:c r="C53" s="42"/>
+      <x:c r="D53" s="42"/>
+      <x:c r="E53" s="42"/>
+      <x:c r="F53" s="42"/>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="41"/>
+      <x:c r="B54" s="41"/>
+      <x:c r="C54" s="42"/>
+      <x:c r="D54" s="42"/>
+      <x:c r="E54" s="42"/>
+      <x:c r="F54" s="42"/>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="41" t="str">
+        <x:v>Health: gradient norm</x:v>
+      </x:c>
+      <x:c r="B55" s="41" t="str">
+        <x:v>base-s1 parameter</x:v>
+      </x:c>
+      <x:c r="C55" s="42" t="str">
+        <x:v>value</x:v>
+      </x:c>
+      <x:c r="D55" s="42" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="E55" s="42"/>
+      <x:c r="F55" s="42"/>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="41" t="str">
+        <x:v>Gradient norm</x:v>
+      </x:c>
+      <x:c r="B56" s="41" t="str">
+        <x:v>net.0.weight</x:v>
+      </x:c>
+      <x:c r="C56" s="42" t="n">
+        <x:v>0.9022008776664734</x:v>
+      </x:c>
+      <x:c r="D56" s="42" t="str">
+        <x:v>health_checks.json</x:v>
+      </x:c>
+      <x:c r="E56" s="42"/>
+      <x:c r="F56" s="42"/>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="41" t="str">
+        <x:v>Gradient norm</x:v>
+      </x:c>
+      <x:c r="B57" s="41" t="str">
+        <x:v>net.0.bias</x:v>
+      </x:c>
+      <x:c r="C57" s="42" t="n">
+        <x:v>0.39315465092658997</x:v>
+      </x:c>
+      <x:c r="D57" s="42" t="str">
+        <x:v>health_checks.json</x:v>
+      </x:c>
+      <x:c r="E57" s="42"/>
+      <x:c r="F57" s="42"/>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="41" t="str">
+        <x:v>Gradient norm</x:v>
+      </x:c>
+      <x:c r="B58" s="41" t="str">
+        <x:v>net.2.weight</x:v>
+      </x:c>
+      <x:c r="C58" s="42" t="n">
+        <x:v>2.77693247795105</x:v>
+      </x:c>
+      <x:c r="D58" s="42" t="str">
+        <x:v>health_checks.json</x:v>
+      </x:c>
+      <x:c r="E58" s="42"/>
+      <x:c r="F58" s="42"/>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="A59" s="41" t="str">
+        <x:v>Gradient norm</x:v>
+      </x:c>
+      <x:c r="B59" s="41" t="str">
+        <x:v>net.2.bias</x:v>
+      </x:c>
+      <x:c r="C59" s="42" t="n">
+        <x:v>0.5370684862136841</x:v>
+      </x:c>
+      <x:c r="D59" s="42" t="str">
+        <x:v>health_checks.json</x:v>
+      </x:c>
+      <x:c r="E59" s="42"/>
+      <x:c r="F59" s="42"/>
+    </x:row>
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="A60" s="41" t="str">
+        <x:v>Gradient norm</x:v>
+      </x:c>
+      <x:c r="B60" s="41" t="str">
+        <x:v>net.4.weight</x:v>
+      </x:c>
+      <x:c r="C60" s="42" t="n">
+        <x:v>2.4162042140960693</x:v>
+      </x:c>
+      <x:c r="D60" s="42" t="str">
+        <x:v>health_checks.json</x:v>
+      </x:c>
+      <x:c r="E60" s="42"/>
+      <x:c r="F60" s="42"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>Gradient norm</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>net.4.bias</x:v>
+      </x:c>
+      <x:c r="C61" s="50" t="n">
+        <x:v>0.6395001411437988</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>health_checks.json</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>